<commit_message>
Release v1.1.0: shared verdict, channels, more scenarios, HARICA TLS fix
- Shared verdict + 35 scenarios grouped DSC/Shared/Not-DSC; Core Facilities, EMBL-EBI and IT-first data-transfer cases
- Explore Channels tab + topic-matched channels in reveals; reveals show example people, not the whole team
- Ingress TLS via cert-manager harica-issuer; versioned image (tag-built) and deploy pinned to v1.1.0
</commit_message>
<xml_diff>
--- a/dsc-catalog.xlsx
+++ b/dsc-catalog.xlsx
@@ -470,7 +470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -581,7 +581,7 @@
         <v>modis</v>
       </c>
       <c r="B5" t="str">
-        <v>MODIS — Multimodal Open Data Integration Support</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="C5" t="str">
         <v>dsc</v>
@@ -706,16 +706,68 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>core-facilities</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Core Facilities</v>
+      </c>
+      <c r="C10" t="str">
+        <v>external</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v>Generating the data — Genomics (GeneCore), Proteomics, Metabolomics, Electron Microscopy, Flow Cytometry and more.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>https://www.embl.org/about/info/core-facilities/</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>embl-ebi</v>
+      </c>
+      <c r="B11" t="str">
+        <v>EMBL-EBI</v>
+      </c>
+      <c r="C11" t="str">
+        <v>external</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v>Public data resources and archives — ArrayExpress, PRIDE, BioStudies, UniProt, Ensembl and more.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>https://www.ebi.ac.uk</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -803,7 +855,7 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="F4" t="str">
-        <v>community, training, leadership</v>
+        <v>training, community, leadership</v>
       </c>
       <c r="G4" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60036724.jpg?itok=KkcLm7zQ</v>
@@ -849,7 +901,7 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="F6" t="str">
-        <v>community</v>
+        <v>training, community</v>
       </c>
       <c r="G6" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60101075.jpg?itok=yAUlN6T3</v>
@@ -872,7 +924,7 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="F7" t="str">
-        <v>modeling, statistics</v>
+        <v>statistics, modeling, training</v>
       </c>
       <c r="G7" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60026366.jpg?itok=1L1JT6Zs</v>
@@ -895,7 +947,7 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="F8" t="str">
-        <v>statistics, software</v>
+        <v>statistics, workflows, training</v>
       </c>
       <c r="G8" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60041652.jpg?itok=uaBzvsJ3</v>
@@ -941,7 +993,7 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="F10" t="str">
-        <v>training</v>
+        <v>machine-learning, training, community</v>
       </c>
       <c r="G10" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60044622.jpg?itok=lPLNMAY6</v>
@@ -964,7 +1016,7 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="F11" t="str">
-        <v>community, software, training</v>
+        <v>training, community, infrastructure</v>
       </c>
       <c r="G11" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60022244.jpg?itok=goRi_n6M</v>
@@ -987,7 +1039,7 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="F12" t="str">
-        <v>modeling</v>
+        <v>statistics, modeling, training</v>
       </c>
       <c r="G12" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60100952.jpg?itok=hyp9yTxB</v>
@@ -1010,7 +1062,7 @@
         <v>Bioimage Analysis Service</v>
       </c>
       <c r="F13" t="str">
-        <v>image-analysis, leadership</v>
+        <v>image-analysis, workflows, training, leadership</v>
       </c>
       <c r="G13" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60005645.jpg?itok=96bzWDuh</v>
@@ -1033,7 +1085,7 @@
         <v>Bioimage Analysis Service</v>
       </c>
       <c r="F14" t="str">
-        <v>image-analysis</v>
+        <v>image-analysis, workflows, software</v>
       </c>
       <c r="G14" t="str">
         <v/>
@@ -1056,7 +1108,7 @@
         <v>Bioimage Analysis Service</v>
       </c>
       <c r="F15" t="str">
-        <v>software, image-analysis, machine-learning</v>
+        <v>image-analysis, workflows, infrastructure</v>
       </c>
       <c r="G15" t="str">
         <v/>
@@ -1079,7 +1131,7 @@
         <v>Bioimage Analysis Service</v>
       </c>
       <c r="F16" t="str">
-        <v>image-analysis, machine-learning, data-management, statistics</v>
+        <v>image-analysis, data-management, infrastructure</v>
       </c>
       <c r="G16" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60008447.jpg?itok=wYk7uKHO</v>
@@ -1102,7 +1154,7 @@
         <v>Bioimage Analysis Service</v>
       </c>
       <c r="F17" t="str">
-        <v>software, image-analysis</v>
+        <v>image-analysis, machine-learning, software</v>
       </c>
       <c r="G17" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60100285.jpg?itok=bPkTsJtR</v>
@@ -1125,7 +1177,7 @@
         <v>Data Management</v>
       </c>
       <c r="F18" t="str">
-        <v>data-management, leadership</v>
+        <v>image-analysis, data-management, data-integration, leadership</v>
       </c>
       <c r="G18" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60100500.jpg?itok=PQgVMvmw</v>
@@ -1148,7 +1200,7 @@
         <v>Data Management</v>
       </c>
       <c r="F19" t="str">
-        <v>data-management, software</v>
+        <v>data-management, software, data-integration</v>
       </c>
       <c r="G19" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60044184.jpg?itok=NaMbcwuX</v>
@@ -1171,7 +1223,7 @@
         <v>Data Management</v>
       </c>
       <c r="F20" t="str">
-        <v>data-management, software</v>
+        <v>data-management, workflows, community</v>
       </c>
       <c r="G20" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60034623.jpg?itok=v-f-IreS</v>
@@ -1194,7 +1246,7 @@
         <v>Data Management</v>
       </c>
       <c r="F21" t="str">
-        <v>data-management, image-analysis, statistics</v>
+        <v>image-analysis, data-management, data-integration</v>
       </c>
       <c r="G21" t="str">
         <v/>
@@ -1214,10 +1266,10 @@
         <v>modis</v>
       </c>
       <c r="E22" t="str">
-        <v>MODIS — Multimodal Open Data Integration Support</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="F22" t="str">
-        <v>data-integration, workflows, leadership</v>
+        <v>data-management, workflows, data-integration, leadership</v>
       </c>
       <c r="G22" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60002771.jpg?itok=Zh7yV9sG</v>
@@ -1237,7 +1289,7 @@
         <v>modis</v>
       </c>
       <c r="E23" t="str">
-        <v>MODIS — Multimodal Open Data Integration Support</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="F23" t="str">
         <v>workflows, software, web</v>
@@ -1260,10 +1312,10 @@
         <v>modis</v>
       </c>
       <c r="E24" t="str">
-        <v>MODIS — Multimodal Open Data Integration Support</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="F24" t="str">
-        <v>software, web</v>
+        <v>software, web, infrastructure</v>
       </c>
       <c r="G24" t="str">
         <v/>
@@ -1271,53 +1323,99 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>thomas-weber</v>
+        <v>laurent-thomas</v>
       </c>
       <c r="B25" t="str">
-        <v>Thomas Weber</v>
+        <v>Laurent Thomas</v>
       </c>
       <c r="C25" t="str">
-        <v>Research Fellow (ARISE)</v>
+        <v>Postdoctoral Fellow</v>
       </c>
       <c r="D25" t="str">
-        <v>fellows</v>
+        <v>modis</v>
       </c>
       <c r="E25" t="str">
-        <v>Fellows</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="F25" t="str">
-        <v>research</v>
+        <v>data-management, workflows, software</v>
       </c>
       <c r="G25" t="str">
-        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60038718.jpg?itok=eQBkIfeV</v>
+        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60100234.jpg?itok=YcuvTUVB</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>marco-wetter</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Marco Wetter</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="D26" t="str">
+        <v>modis</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Multimodal Open Data Integration Support</v>
+      </c>
+      <c r="F26" t="str">
+        <v>software, web, infrastructure</v>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>thomas-weber</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Thomas Weber</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Scientific Workflows Developer</v>
+      </c>
+      <c r="D27" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Data Management</v>
+      </c>
+      <c r="F27" t="str">
+        <v>workflows, software, infrastructure</v>
+      </c>
+      <c r="G27" t="str">
+        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60038718.jpg?itok=eQBkIfeV</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
         <v>nina-habermann</v>
       </c>
-      <c r="B26" t="str">
+      <c r="B28" t="str">
         <v>Nina Habermann</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C28" t="str">
         <v>Operations Manager Data Science Centre</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D28" t="str">
         <v>management</v>
       </c>
-      <c r="E26" t="str">
+      <c r="E28" t="str">
         <v>Management</v>
       </c>
-      <c r="F26" t="str">
-        <v>operations</v>
-      </c>
-      <c r="G26" t="str">
+      <c r="F28" t="str">
+        <v>leadership, operations</v>
+      </c>
+      <c r="G28" t="str">
         <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60020866.jpg?itok=D2zPfuft</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1387,7 +1485,7 @@
         <v>software</v>
       </c>
       <c r="B8" t="str">
-        <v>Research software</v>
+        <v>Software engineering</v>
       </c>
     </row>
     <row r="9">
@@ -1395,7 +1493,7 @@
         <v>web</v>
       </c>
       <c r="B9" t="str">
-        <v>Web &amp; dashboards</v>
+        <v>Web development</v>
       </c>
     </row>
     <row r="10">
@@ -1440,10 +1538,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>research</v>
+        <v>infrastructure</v>
       </c>
       <c r="B15" t="str">
-        <v>Research</v>
+        <v>Infrastructure</v>
       </c>
     </row>
   </sheetData>
@@ -2006,7 +2104,7 @@
         <v>modis</v>
       </c>
       <c r="D6" t="str">
-        <v>MODIS — Multimodal Open Data Integration Support</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="E6" t="str">
         <v>Get access to JupyterHub, BAND, Galaxy and other shared platforms.</v>
@@ -2024,7 +2122,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:L36"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2046,15 +2144,21 @@
         <v>team_name</v>
       </c>
       <c r="G1" t="str">
+        <v>team_also</v>
+      </c>
+      <c r="H1" t="str">
+        <v>team_also_name</v>
+      </c>
+      <c r="I1" t="str">
         <v>needs</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>people</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>why</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>difficulty</v>
       </c>
     </row>
@@ -2066,7 +2170,7 @@
         <v>fellow</v>
       </c>
       <c r="C2" t="str">
-        <v>I have 10,000 microscopy images and need to count the cells in all of them.</v>
+        <v>I've got 10,000 microscopy images and a manual cell-counting habit that's slowly destroying my sanity (and my clicking finger).</v>
       </c>
       <c r="D2" t="str">
         <v>yes</v>
@@ -2078,15 +2182,21 @@
         <v>Bioimage Analysis Service</v>
       </c>
       <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
         <v>image-analysis</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
       </c>
-      <c r="I2" t="str">
-        <v>Counting cells across thousands of images is core bioimage-analysis work.</v>
-      </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
+        <v>Counting cells across thousands of images is bread-and-butter bioimage analysis — and far kinder to your tendons.</v>
+      </c>
+      <c r="L2" t="str">
         <v>easy</v>
       </c>
     </row>
@@ -2098,7 +2208,7 @@
         <v>fellow</v>
       </c>
       <c r="C3" t="str">
-        <v>I ran an experiment with three conditions and don't know which statistical test to use.</v>
+        <v>Three conditions, a pile of data, and absolutely no idea whether it's a t-test, ANOVA, or vibes.</v>
       </c>
       <c r="D3" t="str">
         <v>yes</v>
@@ -2110,15 +2220,21 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
         <v>statistics</v>
       </c>
-      <c r="H3" t="str">
-        <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Choosing and interpreting a statistical test is exactly what the internal support team's statisticians help with.</v>
-      </c>
       <c r="J3" t="str">
+        <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Yuhong Liu</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Picking and interpreting the right statistical test is exactly what the internal support statisticians are for — before you commit to vibes.</v>
+      </c>
+      <c r="L3" t="str">
         <v>easy</v>
       </c>
     </row>
@@ -2130,7 +2246,7 @@
         <v>staff</v>
       </c>
       <c r="C4" t="str">
-        <v>My analysis takes days on my laptop — can I run it as a proper pipeline on the cluster?</v>
+        <v>My analysis takes three days on my laptop, which is now also my space heater. Can we make it a real pipeline on the cluster?</v>
       </c>
       <c r="D4" t="str">
         <v>yes</v>
@@ -2139,18 +2255,24 @@
         <v>modis</v>
       </c>
       <c r="F4" t="str">
-        <v>MODIS — Multimodal Open Data Integration Support</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
         <v>workflows</v>
       </c>
-      <c r="H4" t="str">
-        <v>Charles Girardot, Matthias Monfort</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Turning an analysis into a scalable, reproducible workflow is MODIS / workflow-management territory.</v>
-      </c>
       <c r="J4" t="str">
+        <v>Charles Girardot, Matthias Monfort, Laurent Thomas</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Turning a slow laptop script into a scalable, reproducible cluster workflow is MODIS / workflow-management territory.</v>
+      </c>
+      <c r="L4" t="str">
         <v>easy</v>
       </c>
     </row>
@@ -2162,7 +2284,7 @@
         <v>PI</v>
       </c>
       <c r="C5" t="str">
-        <v>My lab's data is scattered across messy spreadsheets and nobody can find anything.</v>
+        <v>My lab's data lives in 47 spreadsheets named after their authors' moods, and nobody can find last year's results.</v>
       </c>
       <c r="D5" t="str">
         <v>yes</v>
@@ -2174,15 +2296,21 @@
         <v>Data Management</v>
       </c>
       <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
         <v>data-management</v>
       </c>
-      <c r="H5" t="str">
+      <c r="J5" t="str">
         <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
       </c>
-      <c r="I5" t="str">
-        <v>Structuring, documenting and sharing a lab's data is data-management work — often mistaken for an IT problem.</v>
-      </c>
-      <c r="J5" t="str">
+      <c r="K5" t="str">
+        <v>Structuring, documenting and sharing a lab's data is data-management work — frequently mistaken for an IT problem.</v>
+      </c>
+      <c r="L5" t="str">
         <v>boundary</v>
       </c>
     </row>
@@ -2194,7 +2322,7 @@
         <v>fellow</v>
       </c>
       <c r="C6" t="str">
-        <v>I want to train a model to automatically classify cell phenotypes from my images.</v>
+        <v>I want a model to tell apart my cell phenotypes automatically, because my eyes give up around image number 300.</v>
       </c>
       <c r="D6" t="str">
         <v>yes</v>
@@ -2206,15 +2334,21 @@
         <v>Bioimage Analysis Service</v>
       </c>
       <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
         <v>machine-learning, image-analysis</v>
       </c>
-      <c r="H6" t="str">
+      <c r="J6" t="str">
         <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
       </c>
-      <c r="I6" t="str">
-        <v>Training a model to classify phenotypes from images combines machine learning with bioimage analysis.</v>
-      </c>
-      <c r="J6" t="str">
+      <c r="K6" t="str">
+        <v>Training a model to classify phenotypes from images combines machine learning with bioimage analysis — both squarely DSC.</v>
+      </c>
+      <c r="L6" t="str">
         <v>easy</v>
       </c>
     </row>
@@ -2226,7 +2360,7 @@
         <v>PI</v>
       </c>
       <c r="C7" t="str">
-        <v>How many biological replicates do I actually need for this experiment?</v>
+        <v>How many biological replicates do I actually need — asking for the reviewer who will definitely complain about n=3?</v>
       </c>
       <c r="D7" t="str">
         <v>yes</v>
@@ -2238,15 +2372,21 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
         <v>statistics</v>
       </c>
-      <c r="H7" t="str">
-        <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider</v>
-      </c>
-      <c r="I7" t="str">
-        <v>How many replicates you need is a power-analysis question for the statisticians — best asked before you run the experiment.</v>
-      </c>
       <c r="J7" t="str">
+        <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Yuhong Liu</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Replicate numbers are a power-analysis question for the statisticians — best asked before you run the experiment, not after the reviewer does.</v>
+      </c>
+      <c r="L7" t="str">
         <v>boundary</v>
       </c>
     </row>
@@ -2258,7 +2398,7 @@
         <v>core-facility</v>
       </c>
       <c r="C8" t="str">
-        <v>I need to measure the volume of organoids in 3D light-sheet stacks.</v>
+        <v>I need the volume of every organoid in these 3D light-sheet stacks, and counting voxels by hand is not the retirement plan I had in mind.</v>
       </c>
       <c r="D8" t="str">
         <v>yes</v>
@@ -2270,15 +2410,21 @@
         <v>Bioimage Analysis Service</v>
       </c>
       <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
         <v>image-analysis</v>
       </c>
-      <c r="H8" t="str">
+      <c r="J8" t="str">
         <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
       </c>
-      <c r="I8" t="str">
+      <c r="K8" t="str">
         <v>Segmenting and measuring structures in 3D microscopy volumes is advanced image analysis.</v>
       </c>
-      <c r="J8" t="str">
+      <c r="L8" t="str">
         <v>easy</v>
       </c>
     </row>
@@ -2290,7 +2436,7 @@
         <v>fellow</v>
       </c>
       <c r="C9" t="str">
-        <v>My Python analysis script works but is painfully slow — can someone help speed it up?</v>
+        <v>My Python script works, technically — I just have time to make coffee, drink it, and regret things while it runs. Can someone speed it up?</v>
       </c>
       <c r="D9" t="str">
         <v>yes</v>
@@ -2302,27 +2448,33 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="G9" t="str">
-        <v>software</v>
+        <v/>
       </c>
       <c r="H9" t="str">
-        <v>Felix Schneider, Renato Alves</v>
+        <v/>
       </c>
       <c r="I9" t="str">
-        <v>Profiling and optimising research code is research-software-engineering help.</v>
+        <v>workflows</v>
       </c>
       <c r="J9" t="str">
+        <v>Felix Schneider</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Profiling and optimising research code is research-software-engineering help from the internal support team.</v>
+      </c>
+      <c r="L9" t="str">
         <v>boundary</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>deposit-data</v>
+        <v>metadata-standards</v>
       </c>
       <c r="B10" t="str">
         <v>fellow</v>
       </c>
       <c r="C10" t="str">
-        <v>A journal wants me to deposit my data in a public repository before publishing.</v>
+        <v>A consortium insists my dataset follow "community metadata standards", which sounds important and means absolutely nothing to me right now.</v>
       </c>
       <c r="D10" t="str">
         <v>yes</v>
@@ -2334,16 +2486,22 @@
         <v>Data Management</v>
       </c>
       <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
         <v>data-management</v>
       </c>
-      <c r="H10" t="str">
+      <c r="J10" t="str">
         <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
       </c>
-      <c r="I10" t="str">
-        <v>Choosing the right repository and making data FAIR is a data-management service.</v>
-      </c>
-      <c r="J10" t="str">
-        <v>easy</v>
+      <c r="K10" t="str">
+        <v>Translating "community metadata standards" into actual ontologies and fields is exactly what the Data Management team does — so your data plays nicely with everyone else's.</v>
+      </c>
+      <c r="L10" t="str">
+        <v>boundary</v>
       </c>
     </row>
     <row r="11">
@@ -2354,7 +2512,7 @@
         <v>PI</v>
       </c>
       <c r="C11" t="str">
-        <v>My grant application needs a data management plan and I don't know where to start.</v>
+        <v>My grant needs a data management plan, the deadline is Friday, and "I'll keep it on my laptop" apparently isn't one.</v>
       </c>
       <c r="D11" t="str">
         <v>yes</v>
@@ -2366,15 +2524,21 @@
         <v>Data Management</v>
       </c>
       <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
         <v>data-management</v>
       </c>
-      <c r="H11" t="str">
+      <c r="J11" t="str">
         <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
       </c>
-      <c r="I11" t="str">
-        <v>Writing the data management plan for a grant is a core data-management service.</v>
-      </c>
-      <c r="J11" t="str">
+      <c r="K11" t="str">
+        <v>Writing the data management plan for a grant is a core data-management service — ideally before Friday.</v>
+      </c>
+      <c r="L11" t="str">
         <v>easy</v>
       </c>
     </row>
@@ -2386,7 +2550,7 @@
         <v>fellow</v>
       </c>
       <c r="C12" t="str">
-        <v>I'd like to learn enough Python to analyse my own data.</v>
+        <v>I'd like to learn just enough Python to analyse my own data and stop bribing the postdoc next door with cake.</v>
       </c>
       <c r="D12" t="str">
         <v>yes</v>
@@ -2398,15 +2562,21 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
         <v>training</v>
       </c>
-      <c r="H12" t="str">
-        <v>Lisanna Paladin, Sarah Kaspar, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves</v>
-      </c>
-      <c r="I12" t="str">
-        <v>Learning to code for data analysis is covered by the Data Science Centre's training offer.</v>
-      </c>
       <c r="J12" t="str">
+        <v>Lisanna Paladin, Sarah Kaspar, Deborah Udoh, Eva-Maria Geissen, Felix Schneider, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves, Yuhong Liu</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Learning to code for data analysis is covered by the Data Science Centre's training offer — cake optional.</v>
+      </c>
+      <c r="L12" t="str">
         <v>easy</v>
       </c>
     </row>
@@ -2418,7 +2588,7 @@
         <v>staff</v>
       </c>
       <c r="C13" t="str">
-        <v>Our analysis code is a mess of files called final_v3_REALLY_final.py — how do we manage it properly?</v>
+        <v>Our codebase is fifteen files called final_v3_REALLY_final.py and we honestly don't know which one runs. Help?</v>
       </c>
       <c r="D13" t="str">
         <v>yes</v>
@@ -2430,36 +2600,42 @@
         <v>Data Science Internal Support</v>
       </c>
       <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
         <v>software, training</v>
       </c>
-      <c r="H13" t="str">
-        <v>Lisanna Paladin, Sarah Kaspar, Felix Schneider, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves</v>
-      </c>
-      <c r="I13" t="str">
-        <v>Setting up version control and good software practice is research-software-engineering help.</v>
-      </c>
       <c r="J13" t="str">
+        <v>Lisanna Paladin, Sarah Kaspar, Deborah Udoh, Eva-Maria Geissen, Felix Schneider, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves, Yuhong Liu</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Setting up version control and sane software practice is research-software-engineering help from the internal support team.</v>
+      </c>
+      <c r="L13" t="str">
         <v>boundary</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>gpu-server</v>
+        <v>count-the-dots</v>
       </c>
       <c r="B14" t="str">
-        <v>PI</v>
+        <v>core-facility</v>
       </c>
       <c r="C14" t="str">
-        <v>I need a powerful GPU machine to train my deep-learning models.</v>
+        <v>I have a beautiful confocal stack and just need someone to count the fluorescent puncta per nucleus — automatically, for 500 images.</v>
       </c>
       <c r="D14" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="E14" t="str">
-        <v>it-services</v>
+        <v>bioimage-analysis</v>
       </c>
       <c r="F14" t="str">
-        <v>IT Services</v>
+        <v>Bioimage Analysis Service</v>
       </c>
       <c r="G14" t="str">
         <v/>
@@ -2468,30 +2644,36 @@
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>Buying and running GPU hardware is IT. Designing and training the model itself is the DSC — so come to us once the machine exists.</v>
+        <v>image-analysis</v>
       </c>
       <c r="J14" t="str">
-        <v>boundary</v>
+        <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Automated puncta detection and per-nucleus quantification across hundreds of images is exactly what the Bioimage Analysis Service does.</v>
+      </c>
+      <c r="L14" t="str">
+        <v>easy</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>cluster-account</v>
+        <v>shiny-deploy</v>
       </c>
       <c r="B15" t="str">
         <v>fellow</v>
       </c>
       <c r="C15" t="str">
-        <v>I can't log in to the HPC cluster — my account isn't working.</v>
+        <v>I built an R Shiny app to explore our results and my collaborators keep asking me to "just send the link" — can someone host it properly instead of me leaving my laptop on overnight?</v>
       </c>
       <c r="D15" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="E15" t="str">
-        <v>it-services</v>
+        <v>modis</v>
       </c>
       <c r="F15" t="str">
-        <v>IT Services</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="G15" t="str">
         <v/>
@@ -2500,30 +2682,36 @@
         <v/>
       </c>
       <c r="I15" t="str">
-        <v>Accounts and access are managed by IT. How to actually run your analysis on the cluster is the DSC.</v>
+        <v>web, software</v>
       </c>
       <c r="J15" t="str">
+        <v>Matthias Monfort, Nayeem Reza, Laurent Thomas, Marco Wetter</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Deploying and hosting containerised interactive apps (Shiny, dashboards) on EMBL infrastructure is MODIS's ShinyProxy territory — so your laptop can finally sleep.</v>
+      </c>
+      <c r="L15" t="str">
         <v>boundary</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>matlab-license</v>
+        <v>harmonise-metadata</v>
       </c>
       <c r="B16" t="str">
-        <v>staff</v>
+        <v>PI</v>
       </c>
       <c r="C16" t="str">
-        <v>I need a MATLAB licence installed so I can run an analysis script.</v>
+        <v>I have five old datasets whose sample sheets each invented their own words for "timepoint" and "treatment", and I need them to line up so I can analyse them together.</v>
       </c>
       <c r="D16" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="E16" t="str">
-        <v>it-services</v>
+        <v>data-management</v>
       </c>
       <c r="F16" t="str">
-        <v>IT Services</v>
+        <v>Data Management</v>
       </c>
       <c r="G16" t="str">
         <v/>
@@ -2532,30 +2720,36 @@
         <v/>
       </c>
       <c r="I16" t="str">
-        <v>Software licences and installation are handled by IT — even when the software is for data analysis.</v>
+        <v>data-management, data-integration</v>
       </c>
       <c r="J16" t="str">
+        <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Harmonising inconsistent metadata into one coherent, integrable schema is exactly what the Data Management team does — so "t0", "0h" and "baseline" finally mean the same thing.</v>
+      </c>
+      <c r="L16" t="str">
         <v>boundary</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>database-server</v>
+        <v>containerise-pipeline</v>
       </c>
       <c r="B17" t="str">
-        <v>PI</v>
+        <v>staff</v>
       </c>
       <c r="C17" t="str">
-        <v>Can you set up a database server to hold my lab's data?</v>
+        <v>My analysis pipeline runs perfectly on my machine and absolutely nowhere else — I'd like to containerise it so reviewers (and future me) can actually reproduce it.</v>
       </c>
       <c r="D17" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="E17" t="str">
-        <v>it-services</v>
+        <v>modis</v>
       </c>
       <c r="F17" t="str">
-        <v>IT Services</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="G17" t="str">
         <v/>
@@ -2564,21 +2758,27 @@
         <v/>
       </c>
       <c r="I17" t="str">
-        <v>Hosting and maintaining a database server is IT infrastructure. Structuring the data and making it FAIR is the DSC's Data Management team.</v>
+        <v>workflows, software</v>
       </c>
       <c r="J17" t="str">
+        <v>Charles Girardot, Matthias Monfort, Nayeem Reza, Laurent Thomas, Marco Wetter</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Containerising a pipeline for portability and reproducibility is core MODIS / workflow work — defeating the eternal "works on my machine" curse.</v>
+      </c>
+      <c r="L17" t="str">
         <v>boundary</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>shared-drive</v>
+        <v>gpu-server</v>
       </c>
       <c r="B18" t="str">
-        <v>staff</v>
+        <v>PI</v>
       </c>
       <c r="C18" t="str">
-        <v>Our shared network drive is full and I can't save my results.</v>
+        <v>I need a beast of a GPU machine to train my deep-learning model before the heat death of the universe.</v>
       </c>
       <c r="D18" t="str">
         <v>no</v>
@@ -2596,21 +2796,27 @@
         <v/>
       </c>
       <c r="I18" t="str">
-        <v>Storage capacity and network drives are IT. The DSC can later help you organise and archive what's on them.</v>
+        <v/>
       </c>
       <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v>Buying and racking GPU hardware is IT. We (the DSC) design and train the model once the metal is humming — bring it to us then.</v>
+      </c>
+      <c r="L18" t="str">
         <v>boundary</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>jupyter-down</v>
+        <v>matlab-license</v>
       </c>
       <c r="B19" t="str">
-        <v>fellow</v>
+        <v>staff</v>
       </c>
       <c r="C19" t="str">
-        <v>The shared JupyterHub server keeps crashing.</v>
+        <v>My script demands a MATLAB licence and refuses to run without one. Send help.</v>
       </c>
       <c r="D19" t="str">
         <v>no</v>
@@ -2628,21 +2834,27 @@
         <v/>
       </c>
       <c r="I19" t="str">
-        <v>Keeping the server infrastructure running is IT. Help writing or fixing the notebooks themselves is the DSC.</v>
+        <v/>
       </c>
       <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v>Software licences and installation are IT's department — even when the software is pure data crunching. We can't conjure you a licence, sorry.</v>
+      </c>
+      <c r="L19" t="str">
         <v>boundary</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>remote-access</v>
+        <v>shared-drive</v>
       </c>
       <c r="B20" t="str">
-        <v>fellow</v>
+        <v>staff</v>
       </c>
       <c r="C20" t="str">
-        <v>I can't reach my data on the institute server when I work from home.</v>
+        <v>Our shared network drive is full and my results have nowhere to live. The dreaded "disk full" strikes again.</v>
       </c>
       <c r="D20" t="str">
         <v>no</v>
@@ -2660,21 +2872,27 @@
         <v/>
       </c>
       <c r="I20" t="str">
-        <v>Remote access and VPN are handled by IT, not the Data Science Centre.</v>
+        <v/>
       </c>
       <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v>Storage capacity and network drives are IT's to grow. The DSC can later help you tidy and archive the mess — but the extra terabytes come from IT.</v>
+      </c>
+      <c r="L20" t="str">
         <v>boundary</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>backups</v>
+        <v>remote-access</v>
       </c>
       <c r="B21" t="str">
-        <v>PI</v>
+        <v>fellow</v>
       </c>
       <c r="C21" t="str">
-        <v>I want automatic backups set up for my project files.</v>
+        <v>Working from home and I can't reach my data on the institute server — the VPN and I are not on speaking terms.</v>
       </c>
       <c r="D21" t="str">
         <v>no</v>
@@ -2692,15 +2910,591 @@
         <v/>
       </c>
       <c r="I21" t="str">
-        <v>Backup infrastructure is IT. Planning long-term data preservation and sharing is the DSC's Data Management team.</v>
+        <v/>
       </c>
       <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v>Remote access and VPN wrangling are IT, not the Data Science Centre. Once you're connected, we're happy to talk data.</v>
+      </c>
+      <c r="L21" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>demux-and-counts</v>
+      </c>
+      <c r="B22" t="str">
+        <v>fellow</v>
+      </c>
+      <c r="C22" t="str">
+        <v>GeneCore sequenced my 96 RNA libraries — now can the DSC demultiplex them, run FastQC, and hand me a tidy gene-count matrix?</v>
+      </c>
+      <c r="D22" t="str">
+        <v>no</v>
+      </c>
+      <c r="E22" t="str">
+        <v>core-facilities</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Core Facilities</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v>Demultiplexing, standard QC reports and a reference-aligned count matrix are GeneCore's standard primary processing, delivered bundled with the run. The DSC only takes over for the custom downstream — differential expression, odd designs, integration.</v>
+      </c>
+      <c r="L22" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>uniprot-lookup</v>
+      </c>
+      <c r="B23" t="str">
+        <v>fellow</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Where do I find out if my protein of interest is already annotated in UniProt?</v>
+      </c>
+      <c r="D23" t="str">
+        <v>no</v>
+      </c>
+      <c r="E23" t="str">
+        <v>embl-ebi</v>
+      </c>
+      <c r="F23" t="str">
+        <v>EMBL-EBI</v>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v>UniProt is an EMBL-EBI public resource — that's where annotations live. The DSC isn't a lookup desk for public databases.</v>
+      </c>
+      <c r="L23" t="str">
+        <v>easy</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>cluster-account</v>
+      </c>
+      <c r="B24" t="str">
+        <v>fellow</v>
+      </c>
+      <c r="C24" t="str">
+        <v>The HPC cluster keeps rejecting my login and I'm starting to take it personally.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E24" t="str">
+        <v>internal-support</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Data Science Internal Support</v>
+      </c>
+      <c r="G24" t="str">
+        <v>it-services</v>
+      </c>
+      <c r="H24" t="str">
+        <v>IT Services</v>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v>Lisanna Paladin, Sarah Kaspar, Deborah Udoh, Eva-Maria Geissen, Felix Schneider, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves, Yuhong Liu</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Come to the DSC first — we'll get you oriented and show you how to actually make the cluster do real analysis, then point you to IT, who own the accounts and SSH keys that unlock access.</v>
+      </c>
+      <c r="L24" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>database-server</v>
+      </c>
+      <c r="B25" t="str">
+        <v>PI</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Can you spin up a database server to hold my lab's ever-growing pile of data?</v>
+      </c>
+      <c r="D25" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E25" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Data Management</v>
+      </c>
+      <c r="G25" t="str">
+        <v>it-services</v>
+      </c>
+      <c r="H25" t="str">
+        <v>IT Services</v>
+      </c>
+      <c r="I25" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Start with the DSC's Data Management team — they advise which database to pick and design a FAIR schema so it isn't chaos. IT then hosts and maintains the actual server (a VM or Kubernetes DB operator).</v>
+      </c>
+      <c r="L25" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>jupyter-down</v>
+      </c>
+      <c r="B26" t="str">
+        <v>fellow</v>
+      </c>
+      <c r="C26" t="str">
+        <v>The shared JupyterHub server keeps crashing right in the middle of my analysis.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E26" t="str">
+        <v>internal-support</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Data Science Internal Support</v>
+      </c>
+      <c r="G26" t="str">
+        <v>it-services</v>
+      </c>
+      <c r="H26" t="str">
+        <v>IT Services</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v>Lisanna Paladin, Sarah Kaspar, Deborah Udoh, Eva-Maria Geissen, Felix Schneider, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves, Yuhong Liu</v>
+      </c>
+      <c r="K26" t="str">
+        <v>The DSC runs and governs the JupyterHub service, so come to us first when it falls over. IT provides the underlying infrastructure it sits on.</v>
+      </c>
+      <c r="L26" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>backups</v>
+      </c>
+      <c r="B27" t="str">
+        <v>PI</v>
+      </c>
+      <c r="C27" t="str">
+        <v>I'd like automatic backups for my project files, ideally before disaster strikes rather than after.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E27" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Data Management</v>
+      </c>
+      <c r="G27" t="str">
+        <v>it-services</v>
+      </c>
+      <c r="H27" t="str">
+        <v>IT Services</v>
+      </c>
+      <c r="I27" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Start with the DSC's Data Management team to plan what's worth keeping and how to preserve and share it long-term. IT then runs the backup infrastructure that copies your bytes.</v>
+      </c>
+      <c r="L27" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>reads-to-pipeline</v>
+      </c>
+      <c r="B28" t="str">
+        <v>PI</v>
+      </c>
+      <c r="C28" t="str">
+        <v>GeneCore is handing me raw reads from a 200-sample study and I need a reproducible pipeline to process all of it.</v>
+      </c>
+      <c r="D28" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E28" t="str">
+        <v>modis</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Multimodal Open Data Integration Support</v>
+      </c>
+      <c r="G28" t="str">
+        <v>core-facilities</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Core Facilities</v>
+      </c>
+      <c r="I28" t="str">
+        <v>workflows, data-management</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Charles Girardot, Matthias Monfort, Laurent Thomas</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Core Facilities deliver the raw reads; MODIS builds the scalable, reproducible pipeline to turn them into results. Two stops, one happy genomicist.</v>
+      </c>
+      <c r="L28" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>maxquant-search</v>
+      </c>
+      <c r="B29" t="str">
+        <v>staff</v>
+      </c>
+      <c r="C29" t="str">
+        <v>My 40 protein samples are off the mass spec — can you run a MaxQuant search and give me identified, quantified proteins? Sounds like a proteomics-bioinformatics job, right?</v>
+      </c>
+      <c r="D29" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E29" t="str">
+        <v>internal-support</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Data Science Internal Support</v>
+      </c>
+      <c r="G29" t="str">
+        <v>core-facilities</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Core Facilities</v>
+      </c>
+      <c r="I29" t="str">
+        <v>statistics, workflows</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Yuhong Liu</v>
+      </c>
+      <c r="K29" t="str">
+        <v>A standard MaxQuant identification-and-quantification search is actually the Proteomics Core Facility's bundled service. Start with the DSC and we'll point you there for the standard search, then pick up the custom bit — bespoke statistics and a reproducible downstream workflow.</v>
+      </c>
+      <c r="L29" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>archive-before-pub</v>
+      </c>
+      <c r="B30" t="str">
+        <v>staff</v>
+      </c>
+      <c r="C30" t="str">
+        <v>My paper's in review and I need to deposit my transcriptomics data in a public archive — which one, and how do I make it FAIR?</v>
+      </c>
+      <c r="D30" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E30" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Data Management</v>
+      </c>
+      <c r="G30" t="str">
+        <v>embl-ebi</v>
+      </c>
+      <c r="H30" t="str">
+        <v>EMBL-EBI</v>
+      </c>
+      <c r="I30" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Data Management helps you pick the right repository and make the data FAIR; EMBL-EBI hosts the archive (e.g. ArrayExpress) that actually stores it. Talk to us first.</v>
+      </c>
+      <c r="L30" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>pipeline-and-dashboard</v>
+      </c>
+      <c r="B31" t="str">
+        <v>PI</v>
+      </c>
+      <c r="C31" t="str">
+        <v>My core-facility output is great but my lab can't explore it — I want a pipeline that feeds an interactive dashboard everyone can click through.</v>
+      </c>
+      <c r="D31" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E31" t="str">
+        <v>modis</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Multimodal Open Data Integration Support</v>
+      </c>
+      <c r="G31" t="str">
+        <v>internal-support</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Data Science Internal Support</v>
+      </c>
+      <c r="I31" t="str">
+        <v>workflows, software</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Charles Girardot, Matthias Monfort, Nayeem Reza, Laurent Thomas, Marco Wetter</v>
+      </c>
+      <c r="K31" t="str">
+        <v>MODIS wires the workflow into a deployable dashboard; Internal Support's RSEs help polish and maintain the app. Goodbye, screenshots pasted into Mattermost.</v>
+      </c>
+      <c r="L31" t="str">
+        <v>hard</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>compound-annotation</v>
+      </c>
+      <c r="B32" t="str">
+        <v>fellow</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Metabolomics ran my samples and gave me annotated compounds, but now I want to correlate those metabolite levels against my custom drug-dose design — can the DSC crunch that?</v>
+      </c>
+      <c r="D32" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E32" t="str">
+        <v>internal-support</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Data Science Internal Support</v>
+      </c>
+      <c r="G32" t="str">
+        <v>core-facilities</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Core Facilities</v>
+      </c>
+      <c r="I32" t="str">
+        <v>statistics</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Yuhong Liu</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Standard compound annotation is the Metabolomics Core Facility's bundled deliverable, so start with the DSC and we'll confirm that part lives there — then we pick up the custom downstream, the dose-response statistics and correlation analysis.</v>
+      </c>
+      <c r="L32" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>flow-gating</v>
+      </c>
+      <c r="B33" t="str">
+        <v>core-facility</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Flow Cytometry already gated my populations the standard way — now I want an unsupervised clustering and trajectory analysis across 80 samples to find a subset nobody's drawn a gate around yet.</v>
+      </c>
+      <c r="D33" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E33" t="str">
+        <v>internal-support</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Data Science Internal Support</v>
+      </c>
+      <c r="G33" t="str">
+        <v>core-facilities</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Core Facilities</v>
+      </c>
+      <c r="I33" t="str">
+        <v>statistics, machine-learning</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Jacobo Miranda, Yuhong Liu</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Standard gating is the Flow Cytometry Core Facility's job; the DSC takes over for the custom bit — unsupervised clustering and high-dimensional analysis that no manual gate can capture. Talk to us first for the downstream.</v>
+      </c>
+      <c r="L33" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>deconvolved-quant</v>
+      </c>
+      <c r="B34" t="str">
+        <v>staff</v>
+      </c>
+      <c r="C34" t="str">
+        <v>The Light Microscopy facility deconvolved and stitched my big tiled acquisition beautifully — now I need a custom pipeline to quantify membrane-to-cytoplasm ratios per cell across the whole mosaic.</v>
+      </c>
+      <c r="D34" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E34" t="str">
+        <v>bioimage-analysis</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Bioimage Analysis Service</v>
+      </c>
+      <c r="G34" t="str">
+        <v>core-facilities</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Core Facilities</v>
+      </c>
+      <c r="I34" t="str">
+        <v>image-analysis</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Acquisition, deconvolution and stitching are the facility's standard processing; bespoke per-cell quantification is DSC bioimage analysis. Come to us first for the custom measurement, then the facility for any reacquisition.</v>
+      </c>
+      <c r="L34" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>collaborator-transfer</v>
+      </c>
+      <c r="B35" t="str">
+        <v>PI</v>
+      </c>
+      <c r="C35" t="str">
+        <v>A collaborator in Japan needs to send us 8 TB of imaging data and email attachments are, shockingly, not up to the task.</v>
+      </c>
+      <c r="D35" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E35" t="str">
+        <v>it-services</v>
+      </c>
+      <c r="F35" t="str">
+        <v>IT Services</v>
+      </c>
+      <c r="G35" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Data Management</v>
+      </c>
+      <c r="I35" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
+      </c>
+      <c r="K35" t="str">
+        <v>IT first — they own the secure large-file transfer (Aspera/Globus) that actually moves 8 TB across the planet. The DSC's Data Management team then helps structure and document what arrives so it isn't 8 TB of mystery.</v>
+      </c>
+      <c r="L35" t="str">
+        <v>boundary</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>site-to-site</v>
+      </c>
+      <c r="B36" t="str">
+        <v>staff</v>
+      </c>
+      <c r="C36" t="str">
+        <v>I need to shuttle a multi-terabyte dataset from EMBL Heidelberg over to EMBL-EBI Hinxton, and dragging it onto a USB stick feels wrong somehow.</v>
+      </c>
+      <c r="D36" t="str">
+        <v>shared</v>
+      </c>
+      <c r="E36" t="str">
+        <v>it-services</v>
+      </c>
+      <c r="F36" t="str">
+        <v>IT Services</v>
+      </c>
+      <c r="G36" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Data Management</v>
+      </c>
+      <c r="I36" t="str">
+        <v>data-management</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Moving data between EMBL sites runs on IT's inter-site transfer infrastructure, so go to IT first. The DSC's Data Management team helps organise and document the dataset so the copy at the other end makes sense.</v>
+      </c>
+      <c r="L36" t="str">
         <v>boundary</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Release v1.2.0: routing model, Consulting/Community, hash routing, logos
- Reframe swipe prompt to "Can the Data Science Centre help with this?"; drop difficulty and pillars.
- Scenario routing tools: teams:, cross_team:, people:, channels:; broaden over-attributed scenarios.
- Reveal: 3 people by default with show-all; simplified shared verdict.
- Explore: Training links to Bio-IT resources; Services -> Consulting (+booking banner); Channels -> Community (+initiatives); real platform logos.
- Lightweight URL-hash routing (refresh/back/forward, shareable Explore/Directory).
- 10 random questions per round.
</commit_message>
<xml_diff>
--- a/dsc-catalog.xlsx
+++ b/dsc-catalog.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Pillars" sheetId="1" r:id="rId1"/>
-    <sheet name="Teams" sheetId="2" r:id="rId2"/>
-    <sheet name="Members" sheetId="3" r:id="rId3"/>
-    <sheet name="Competencies" sheetId="4" r:id="rId4"/>
-    <sheet name="Platforms" sheetId="5" r:id="rId5"/>
-    <sheet name="Training" sheetId="6" r:id="rId6"/>
-    <sheet name="Services" sheetId="7" r:id="rId7"/>
+    <sheet name="Teams" sheetId="1" r:id="rId1"/>
+    <sheet name="Members" sheetId="2" r:id="rId2"/>
+    <sheet name="Competencies" sheetId="3" r:id="rId3"/>
+    <sheet name="Platforms" sheetId="4" r:id="rId4"/>
+    <sheet name="Training" sheetId="5" r:id="rId5"/>
+    <sheet name="Consulting" sheetId="6" r:id="rId6"/>
+    <sheet name="Initiatives" sheetId="7" r:id="rId7"/>
     <sheet name="Scenarios" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:F11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -414,359 +414,227 @@
         <v>name</v>
       </c>
       <c r="C1" t="str">
+        <v>kind</v>
+      </c>
+      <c r="D1" t="str">
         <v>blurb</v>
+      </c>
+      <c r="E1" t="str">
+        <v>link</v>
+      </c>
+      <c r="F1" t="str">
+        <v>ticket</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>training</v>
+        <v>internal-support</v>
       </c>
       <c r="B2" t="str">
-        <v>Training</v>
+        <v>Data Science Internal Support</v>
       </c>
       <c r="C2" t="str">
-        <v>Courses and workshops that build data and software skills.</v>
+        <v>dsc</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Empowering research through consulting, training, community support and infrastructure.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>https://www.embl.org/about/info/data-science-centre/</v>
+      </c>
+      <c r="F2" t="str">
+        <v>https://bio-it.embl.de/datascience-consulting/</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>consulting</v>
+        <v>bioimage-analysis</v>
       </c>
       <c r="B3" t="str">
-        <v>Consulting</v>
+        <v>Bioimage Analysis Service</v>
       </c>
       <c r="C3" t="str">
-        <v>One-to-one expert advice on your data, analysis and methods.</v>
+        <v>dsc</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Reproducible extraction of quantitative information from microscopy data.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>https://www.embl.org/about/info/data-science-centre/</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://bio-it.embl.de/datascience-consulting/</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>community</v>
+        <v>data-management</v>
       </c>
       <c r="B4" t="str">
-        <v>Community</v>
+        <v>Data Management</v>
       </c>
       <c r="C4" t="str">
-        <v>Connecting people, channels and events across EMBL data science.</v>
+        <v>dsc</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Making data workflows easier, more robust and reproducible</v>
+      </c>
+      <c r="E4" t="str">
+        <v>https://www.embl.org/about/info/data-science-centre/</v>
+      </c>
+      <c r="F4" t="str">
+        <v>https://bio-it.embl.de/datascience-consulting/</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>infrastructure</v>
+        <v>modis</v>
       </c>
       <c r="B5" t="str">
-        <v>Infrastructure</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="C5" t="str">
-        <v>Shared platforms, compute and tools for doing the work.</v>
+        <v>dsc</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Solutions and support for FAIR data management, integration and publication.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>https://www.embl.org/about/info/data-science-centre/</v>
+      </c>
+      <c r="F5" t="str">
+        <v>https://bio-it.embl.de/datascience-consulting/</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>chairs</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Chairs</v>
+      </c>
+      <c r="C6" t="str">
+        <v>dsc</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Leadership of the Data Science Centre.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>https://www.embl.org/about/info/data-science-centre/members/</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>management</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Management</v>
+      </c>
+      <c r="C7" t="str">
+        <v>dsc</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Operations and coordination of the Data Science Centre.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>https://www.embl.org/about/info/data-science-centre/members/</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>fellows</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Fellows</v>
+      </c>
+      <c r="C8" t="str">
+        <v>dsc</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Fellows and visiting researchers within the Data Science Centre.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>https://www.embl.org/about/info/data-science-centre/members/</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>it-services</v>
+      </c>
+      <c r="B9" t="str">
+        <v>IT Services</v>
+      </c>
+      <c r="C9" t="str">
+        <v>external</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Hardware, accounts, software licences, storage and network infrastructure.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>https://www.embl.org/about/info/it-services/</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>core-facilities</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Core Facilities</v>
+      </c>
+      <c r="C10" t="str">
+        <v>external</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Data producers, GeneCore, Proteomics, Metabolomics, ALMF, and more.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>https://www.embl.org/services-facilities/</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>embl-ebi</v>
+      </c>
+      <c r="B11" t="str">
+        <v>EMBL-EBI</v>
+      </c>
+      <c r="C11" t="str">
+        <v>external</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Public data resources and archives, BioImage Archive, PRIDE, ENA, Ensembl and more.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>https://www.ebi.ac.uk</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>kind</v>
-      </c>
-      <c r="D1" t="str">
-        <v>pillars</v>
-      </c>
-      <c r="E1" t="str">
-        <v>blurb</v>
-      </c>
-      <c r="F1" t="str">
-        <v>link</v>
-      </c>
-      <c r="G1" t="str">
-        <v>mattermost</v>
-      </c>
-      <c r="H1" t="str">
-        <v>ticket</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>internal-support</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Data Science Internal Support</v>
-      </c>
-      <c r="C2" t="str">
-        <v>dsc</v>
-      </c>
-      <c r="D2" t="str">
-        <v>consulting, training, community, infrastructure</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Consulting, training, community and infrastructure support for EMBL researchers.</v>
-      </c>
-      <c r="F2" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
-      </c>
-      <c r="G2" t="str">
-        <v>https://chat.embl.org/embl/channels/data-science</v>
-      </c>
-      <c r="H2" t="str">
-        <v>https://tickets.embl.org/new?queue=data-science</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>bioimage-analysis</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Bioimage Analysis Service</v>
-      </c>
-      <c r="C3" t="str">
-        <v>dsc</v>
-      </c>
-      <c r="D3" t="str">
-        <v>consulting, infrastructure, training</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Reproducible extraction of quantitative information from microscopy data.</v>
-      </c>
-      <c r="F3" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
-      </c>
-      <c r="G3" t="str">
-        <v>https://chat.embl.org/embl/channels/image-analysis</v>
-      </c>
-      <c r="H3" t="str">
-        <v>https://tickets.embl.org/new?queue=image-analysis</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>data-management</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Data Management</v>
-      </c>
-      <c r="C4" t="str">
-        <v>dsc</v>
-      </c>
-      <c r="D4" t="str">
-        <v>consulting, infrastructure</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Making data workflows easier, more robust, reproducible and FAIR.</v>
-      </c>
-      <c r="F4" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
-      </c>
-      <c r="G4" t="str">
-        <v>https://chat.embl.org/embl/channels/data-management</v>
-      </c>
-      <c r="H4" t="str">
-        <v>https://tickets.embl.org/new?queue=data-management</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>modis</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Multimodal Open Data Integration Support</v>
-      </c>
-      <c r="C5" t="str">
-        <v>dsc</v>
-      </c>
-      <c r="D5" t="str">
-        <v>infrastructure, consulting</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Solutions and support for FAIR data management, integration and publication.</v>
-      </c>
-      <c r="F5" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
-      </c>
-      <c r="G5" t="str">
-        <v>https://chat.embl.org/embl/channels/modis</v>
-      </c>
-      <c r="H5" t="str">
-        <v>https://tickets.embl.org/new?queue=modis</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>chairs</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Chairs</v>
-      </c>
-      <c r="C6" t="str">
-        <v>dsc</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v>Scientific leadership of the Data Science Centre.</v>
-      </c>
-      <c r="F6" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/members/</v>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>management</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Management</v>
-      </c>
-      <c r="C7" t="str">
-        <v>dsc</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v>Operations and coordination of the Data Science Centre.</v>
-      </c>
-      <c r="F7" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/members/</v>
-      </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>fellows</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Fellows</v>
-      </c>
-      <c r="C8" t="str">
-        <v>dsc</v>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v>Fellows and visiting researchers within the Data Science Centre.</v>
-      </c>
-      <c r="F8" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/members/</v>
-      </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>it-services</v>
-      </c>
-      <c r="B9" t="str">
-        <v>IT Services</v>
-      </c>
-      <c r="C9" t="str">
-        <v>external</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9" t="str">
-        <v>Hardware, accounts, software licences, storage and network infrastructure.</v>
-      </c>
-      <c r="F9" t="str">
-        <v>https://www.embl.org/it</v>
-      </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>core-facilities</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Core Facilities</v>
-      </c>
-      <c r="C10" t="str">
-        <v>external</v>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v>Generating the data — Genomics (GeneCore), Proteomics, Metabolomics, Electron Microscopy, Flow Cytometry and more.</v>
-      </c>
-      <c r="F10" t="str">
-        <v>https://www.embl.org/about/info/core-facilities/</v>
-      </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>embl-ebi</v>
-      </c>
-      <c r="B11" t="str">
-        <v>EMBL-EBI</v>
-      </c>
-      <c r="C11" t="str">
-        <v>external</v>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
-        <v>Public data resources and archives — ArrayExpress, PRIDE, BioStudies, UniProt, Ensembl and more.</v>
-      </c>
-      <c r="F11" t="str">
-        <v>https://www.ebi.ac.uk</v>
-      </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G28"/>
   <sheetData>
     <row r="1">
@@ -961,7 +829,7 @@
         <v>Isabela Paredes-Cisneros</v>
       </c>
       <c r="C9" t="str">
-        <v>Project Manager – Learning and Impact Assessment</v>
+        <v>Project Manager, Learning and Impact Assessment</v>
       </c>
       <c r="D9" t="str">
         <v>internal-support</v>
@@ -1122,7 +990,7 @@
         <v>Jean-Karim Hériché</v>
       </c>
       <c r="C16" t="str">
-        <v>Computational Scientist – Bioimage Data Analysis and Management</v>
+        <v>Computational Scientist, Bioimage Data Analysis and Management</v>
       </c>
       <c r="D16" t="str">
         <v>bioimage-analysis</v>
@@ -1254,36 +1122,36 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>charles-girardot</v>
+        <v>thomas-weber</v>
       </c>
       <c r="B22" t="str">
-        <v>Charles Girardot</v>
+        <v>Thomas Weber</v>
       </c>
       <c r="C22" t="str">
-        <v>Head of Multimodal Open Data Integration Support</v>
+        <v>Scientific Workflows Developer</v>
       </c>
       <c r="D22" t="str">
-        <v>modis</v>
+        <v>data-management</v>
       </c>
       <c r="E22" t="str">
-        <v>Multimodal Open Data Integration Support</v>
+        <v>Data Management</v>
       </c>
       <c r="F22" t="str">
-        <v>data-management, workflows, data-integration, leadership</v>
+        <v>workflows, software, infrastructure</v>
       </c>
       <c r="G22" t="str">
-        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60002771.jpg?itok=Zh7yV9sG</v>
+        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60038718.jpg?itok=eQBkIfeV</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>matthias-monfort</v>
+        <v>charles-girardot</v>
       </c>
       <c r="B23" t="str">
-        <v>Matthias Monfort</v>
+        <v>Charles Girardot</v>
       </c>
       <c r="C23" t="str">
-        <v>Web Developer / Workflow Management</v>
+        <v>Head of Multimodal Open Data Integration Support</v>
       </c>
       <c r="D23" t="str">
         <v>modis</v>
@@ -1292,21 +1160,21 @@
         <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="F23" t="str">
-        <v>workflows, software, web</v>
+        <v>data-management, workflows, data-integration, leadership</v>
       </c>
       <c r="G23" t="str">
-        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60018989.jpg?itok=bK7v9CaG</v>
+        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60002771.jpg?itok=Zh7yV9sG</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>nayeem-reza</v>
+        <v>matthias-monfort</v>
       </c>
       <c r="B24" t="str">
-        <v>Nayeem Reza</v>
+        <v>Matthias Monfort</v>
       </c>
       <c r="C24" t="str">
-        <v>Senior Software Engineer</v>
+        <v>Web Developer / Workflow Management</v>
       </c>
       <c r="D24" t="str">
         <v>modis</v>
@@ -1315,21 +1183,21 @@
         <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="F24" t="str">
-        <v>software, web, infrastructure</v>
+        <v>workflows, software, web</v>
       </c>
       <c r="G24" t="str">
-        <v/>
+        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60018989.jpg?itok=bK7v9CaG</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>laurent-thomas</v>
+        <v>nayeem-reza</v>
       </c>
       <c r="B25" t="str">
-        <v>Laurent Thomas</v>
+        <v>Nayeem Reza</v>
       </c>
       <c r="C25" t="str">
-        <v>Postdoctoral Fellow</v>
+        <v>Senior Software Engineer</v>
       </c>
       <c r="D25" t="str">
         <v>modis</v>
@@ -1338,21 +1206,21 @@
         <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="F25" t="str">
-        <v>data-management, workflows, software</v>
+        <v>software, web, infrastructure</v>
       </c>
       <c r="G25" t="str">
-        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60100234.jpg?itok=YcuvTUVB</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>marco-wetter</v>
+        <v>laurent-thomas</v>
       </c>
       <c r="B26" t="str">
-        <v>Marco Wetter</v>
+        <v>Laurent Thomas</v>
       </c>
       <c r="C26" t="str">
-        <v>Full Stack Developer</v>
+        <v>Postdoctoral Fellow</v>
       </c>
       <c r="D26" t="str">
         <v>modis</v>
@@ -1361,33 +1229,33 @@
         <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="F26" t="str">
-        <v>software, web, infrastructure</v>
+        <v>data-management, workflows, software</v>
       </c>
       <c r="G26" t="str">
-        <v/>
+        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60100234.jpg?itok=YcuvTUVB</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>thomas-weber</v>
+        <v>marco-wetter</v>
       </c>
       <c r="B27" t="str">
-        <v>Thomas Weber</v>
+        <v>Marco Wetter</v>
       </c>
       <c r="C27" t="str">
-        <v>Scientific Workflows Developer</v>
+        <v>Full Stack Developer</v>
       </c>
       <c r="D27" t="str">
-        <v>data-management</v>
+        <v>modis</v>
       </c>
       <c r="E27" t="str">
-        <v>Data Management</v>
+        <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="F27" t="str">
-        <v>workflows, software, infrastructure</v>
+        <v>software, web, infrastructure</v>
       </c>
       <c r="G27" t="str">
-        <v>https://content.embl.org/sites/default/files/styles/medium/public/persons/CP-60038718.jpg?itok=eQBkIfeV</v>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1420,7 +1288,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B15"/>
   <sheetData>
@@ -1551,9 +1419,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1566,12 +1434,9 @@
         <v>category</v>
       </c>
       <c r="D1" t="str">
-        <v>pillars</v>
+        <v>blurb</v>
       </c>
       <c r="E1" t="str">
-        <v>blurb</v>
-      </c>
-      <c r="F1" t="str">
         <v>url</v>
       </c>
     </row>
@@ -1586,13 +1451,10 @@
         <v>Compute &amp; desktops</v>
       </c>
       <c r="D2" t="str">
-        <v>infrastructure</v>
+        <v>Browser-based remote desktop with image-analysis tools running on EMBL compute.</v>
       </c>
       <c r="E2" t="str">
-        <v>Browser-based remote desktop with image-analysis tools running on EMBL compute.</v>
-      </c>
-      <c r="F2" t="str">
-        <v>https://github.com/embl-cba/band</v>
+        <v>https://bandv1.denbi.uni-tuebingen.de/#/eosc-landingpage</v>
       </c>
     </row>
     <row r="3">
@@ -1600,19 +1462,16 @@
         <v>jupyterhub</v>
       </c>
       <c r="B3" t="str">
-        <v>JupyterHub on Kubernetes</v>
+        <v>JupyterHub</v>
       </c>
       <c r="C3" t="str">
         <v>Compute &amp; desktops</v>
       </c>
       <c r="D3" t="str">
-        <v>infrastructure</v>
+        <v>Browser-based RStudio, JupyterLab, code-server and virtual desktops with shared compute.</v>
       </c>
       <c r="E3" t="str">
-        <v>Browser-based RStudio, JupyterLab, code-server and virtual desktops with shared compute.</v>
-      </c>
-      <c r="F3" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
+        <v>https://jupyterhub.embl.de/</v>
       </c>
     </row>
     <row r="4">
@@ -1620,231 +1479,231 @@
         <v>galaxy</v>
       </c>
       <c r="B4" t="str">
-        <v>Galaxy</v>
+        <v>Galaxy instance</v>
       </c>
       <c r="C4" t="str">
         <v>Workflows</v>
       </c>
       <c r="D4" t="str">
-        <v>infrastructure, training</v>
+        <v>Galaxy local instance for accessible, reproducible analysis pipelines.</v>
       </c>
       <c r="E4" t="str">
-        <v>Web platform for reproducible, FAIR bioinformatics workflows.</v>
-      </c>
-      <c r="F4" t="str">
-        <v>https://galaxyproject.org/</v>
+        <v>https://galaxy.embl.de/login/start?redirect=%2F</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>workflows</v>
+        <v>shinyportal</v>
       </c>
       <c r="B5" t="str">
-        <v>Scientific workflows (Nextflow, Snakemake)</v>
+        <v>ShinyPortal</v>
       </c>
       <c r="C5" t="str">
-        <v>Workflows</v>
+        <v>Apps &amp; dashboards</v>
       </c>
       <c r="D5" t="str">
-        <v>infrastructure, consulting</v>
+        <v>Host containerised interactive web apps and Shiny dashboards.</v>
       </c>
       <c r="E5" t="str">
-        <v>Reproducible, scalable analysis pipelines.</v>
-      </c>
-      <c r="F5" t="str">
-        <v>https://www.nextflow.io/</v>
+        <v>https://shiny-portal.embl.de/shinyapps/</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>shinyproxy</v>
+        <v>depictio</v>
       </c>
       <c r="B6" t="str">
-        <v>ShinyProxy</v>
+        <v>Depictio</v>
       </c>
       <c r="C6" t="str">
         <v>Apps &amp; dashboards</v>
       </c>
       <c r="D6" t="str">
-        <v>infrastructure</v>
+        <v>Build interactive dashboards from workflow outputs (Nextflow, Snakemake, Galaxy).</v>
       </c>
       <c r="E6" t="str">
-        <v>Host containerised interactive web apps and Shiny dashboards.</v>
-      </c>
-      <c r="F6" t="str">
-        <v>https://www.shinyproxy.io/</v>
+        <v>https://depictio.github.io/depictio-docs/</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>depictio</v>
+        <v>gitlab</v>
       </c>
       <c r="B7" t="str">
-        <v>Depictio</v>
+        <v>GitLab</v>
       </c>
       <c r="C7" t="str">
-        <v>Apps &amp; dashboards</v>
+        <v>Collaboration</v>
       </c>
       <c r="D7" t="str">
-        <v>infrastructure</v>
+        <v>EMBL's self-hosted Git for code, CI/CD and Pages.</v>
       </c>
       <c r="E7" t="str">
-        <v>Build interactive dashboards from workflow outputs (Nextflow, Snakemake, Galaxy).</v>
-      </c>
-      <c r="F7" t="str">
-        <v>https://github.com/depictio/depictio</v>
+        <v>https://git.embl.org/</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>gitlab</v>
+        <v>mattermost</v>
       </c>
       <c r="B8" t="str">
-        <v>GitLab</v>
+        <v>EMBL Chat (Mattermost)</v>
       </c>
       <c r="C8" t="str">
         <v>Collaboration</v>
       </c>
       <c r="D8" t="str">
-        <v>infrastructure, community</v>
+        <v>Team chat and topic channels across EMBL.</v>
       </c>
       <c r="E8" t="str">
-        <v>EMBL's self-hosted Git for code, CI/CD and Pages.</v>
-      </c>
-      <c r="F8" t="str">
-        <v>https://about.gitlab.com/</v>
+        <v>https://chat.embl.org/</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>mattermost</v>
+        <v>hedgedoc</v>
       </c>
       <c r="B9" t="str">
-        <v>EMBL Chat (Mattermost)</v>
+        <v>pad-bio (HedgeDoc)</v>
       </c>
       <c r="C9" t="str">
         <v>Collaboration</v>
       </c>
       <c r="D9" t="str">
-        <v>community</v>
+        <v>Real-time collaborative markdown notes and documentation.</v>
       </c>
       <c r="E9" t="str">
-        <v>Team chat and topic channels across EMBL.</v>
-      </c>
-      <c r="F9" t="str">
-        <v>https://chat.embl.org/</v>
+        <v>https://pad.bio-it.embl.de/</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>hedgedoc</v>
+        <v>limesurvey</v>
       </c>
       <c r="B10" t="str">
-        <v>pad-bio (HedgeDoc)</v>
+        <v>LimeSurvey</v>
       </c>
       <c r="C10" t="str">
         <v>Collaboration</v>
       </c>
       <c r="D10" t="str">
-        <v>community</v>
+        <v>Surveys and feedback collection for events and the community.</v>
       </c>
       <c r="E10" t="str">
-        <v>Real-time collaborative markdown notes and documentation.</v>
-      </c>
-      <c r="F10" t="str">
-        <v>https://hedgedoc.org/</v>
+        <v>https://survey.bio-it.embl.de/</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>limesurvey</v>
+        <v>labid</v>
       </c>
       <c r="B11" t="str">
-        <v>LimeSurvey</v>
+        <v>LabID</v>
       </c>
       <c r="C11" t="str">
-        <v>Collaboration</v>
+        <v>Data management</v>
       </c>
       <c r="D11" t="str">
-        <v>community</v>
+        <v>Lab inventory and data management for samples and datasets.</v>
       </c>
       <c r="E11" t="str">
-        <v>Surveys and feedback collection for events and the community.</v>
-      </c>
-      <c r="F11" t="str">
-        <v>https://www.limesurvey.org/</v>
+        <v>https://labid.embl.org/</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>labid</v>
+        <v>ds-wizard</v>
       </c>
       <c r="B12" t="str">
-        <v>LabID</v>
+        <v>Data Stewardship Wizard</v>
       </c>
       <c r="C12" t="str">
         <v>Data management</v>
       </c>
       <c r="D12" t="str">
-        <v>infrastructure, consulting</v>
+        <v>Build data management plans interactively.</v>
       </c>
       <c r="E12" t="str">
-        <v>Electronic lab notebook, inventory and sample/dataset tracking.</v>
-      </c>
-      <c r="F12" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>ds-wizard</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Data Stewardship Wizard</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Data management</v>
-      </c>
-      <c r="D13" t="str">
-        <v>consulting, training</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Build data management plans interactively.</v>
-      </c>
-      <c r="F13" t="str">
-        <v>https://ds-wizard.org/</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>data-submission</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Data submission support</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Data management</v>
-      </c>
-      <c r="D14" t="str">
-        <v>consulting</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Guidance on depositing data in the right public repository (FAIR).</v>
-      </c>
-      <c r="F14" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
+        <v>https://ds-wizard.embl.org/wizard/</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>blurb</v>
+      </c>
+      <c r="D1" t="str">
+        <v>url</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>upcoming-courses</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Upcoming courses</v>
+      </c>
+      <c r="C2" t="str">
+        <v>What's coming up, register for the next data &amp; software skills courses.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>https://bio-it.embl.de/upcoming-courses/</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>course-catalogue</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Course catalogue</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Browse all courses, upcoming and past, in the Bio-IT course catalogue.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>https://catalogue.bio-it.embl.de/courses/catalogue/</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>course-materials</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Course materials</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Slides, notebooks and exercises from past courses, free to reuse.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>https://bio-it.embl.de/course-materials/</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1854,144 +1713,106 @@
         <v>name</v>
       </c>
       <c r="C1" t="str">
-        <v>pillars</v>
+        <v>blurb</v>
       </c>
       <c r="D1" t="str">
-        <v>blurb</v>
-      </c>
-      <c r="E1" t="str">
         <v>url</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>carpentries</v>
+        <v>cloud-computing</v>
       </c>
       <c r="B2" t="str">
-        <v>Software &amp; Data Carpentries</v>
+        <v>Cloud computing &amp; storage</v>
       </c>
       <c r="C2" t="str">
-        <v>training, community</v>
+        <v>Selecting and provisioning the hardware resources for online apps and datasets.</v>
       </c>
       <c r="D2" t="str">
-        <v>Hands-on workshops in Git, shell, Python and R for reproducible research.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>https://carpentries.org/</v>
+        <v>https://www.embl.org/about/info/data-science-centre/consulting/</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>train-the-trainer</v>
+        <v>computational-biology</v>
       </c>
       <c r="B3" t="str">
-        <v>Train-the-Trainer</v>
+        <v>Computational biology</v>
       </c>
       <c r="C3" t="str">
-        <v>training, community</v>
+        <v>Bioinformatics, command line, scripting, task automation and biocomputing.</v>
       </c>
       <c r="D3" t="str">
-        <v>Learn to teach — curriculum design, facilitation and learner engagement.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
+        <v>https://www.embl.org/about/info/data-science-centre/consulting/</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>experimental-design</v>
+        <v>mathematical-modelling</v>
       </c>
       <c r="B4" t="str">
-        <v>Experimental design</v>
+        <v>Mathematical modelling</v>
       </c>
       <c r="C4" t="str">
-        <v>training, consulting</v>
+        <v>Adopting mathematical modelling techniques and sharing modelling expertise.</v>
       </c>
       <c r="D4" t="str">
-        <v>Plan studies, power and sample size before you run the experiment.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
+        <v>https://www.embl.org/about/info/data-science-centre/consulting/</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>statistical-analysis</v>
+        <v>workflows-data-management</v>
       </c>
       <c r="B5" t="str">
-        <v>Statistical analysis</v>
+        <v>Scientific workflows &amp; data management</v>
       </c>
       <c r="C5" t="str">
-        <v>training, consulting</v>
+        <v>Workflows and best practices for more efficient, reproducible research.</v>
       </c>
       <c r="D5" t="str">
-        <v>Statistical testing, modelling and interpretation of your data.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
+        <v>https://www.embl.org/about/info/data-science-centre/consulting/</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>mathematical-modeling</v>
+        <v>statistical-methods</v>
       </c>
       <c r="B6" t="str">
-        <v>Mathematical modeling</v>
+        <v>Statistical methods</v>
       </c>
       <c r="C6" t="str">
-        <v>training, consulting</v>
+        <v>Data visualisation, experimental design, hypothesis testing and machine learning.</v>
       </c>
       <c r="D6" t="str">
-        <v>Modelling biological systems quantitatively.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
+        <v>https://www.embl.org/about/info/data-science-centre/consulting/</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>cloud-computing</v>
+        <v>image-analysis</v>
       </c>
       <c r="B7" t="str">
-        <v>Cloud computing</v>
+        <v>Image analysis</v>
       </c>
       <c r="C7" t="str">
-        <v>training, infrastructure</v>
+        <v>Extracting meaningful biological information from microscopy data, reproducibly.</v>
       </c>
       <c r="D7" t="str">
-        <v>Containers, web apps and running code on EMBL cloud infrastructure.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>https://www.embl.org/about/info/data-science-centre/</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>management-plans</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Data &amp; software management plans</v>
-      </c>
-      <c r="C8" t="str">
-        <v>training, consulting</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Write data and software management plans, with a guided wizard.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>https://ds-wizard.org/</v>
+        <v>https://www.embl.org/about/info/data-science-centre/consulting/</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:D6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2001,121 +1822,85 @@
         <v>name</v>
       </c>
       <c r="C1" t="str">
-        <v>team</v>
+        <v>blurb</v>
       </c>
       <c r="D1" t="str">
-        <v>team_name</v>
-      </c>
-      <c r="E1" t="str">
-        <v>blurb</v>
-      </c>
-      <c r="F1" t="str">
-        <v>link</v>
+        <v>url</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>consulting</v>
+        <v>epug</v>
       </c>
       <c r="B2" t="str">
-        <v>Data science consulting</v>
+        <v>EMBL Python User Group (EPUG)</v>
       </c>
       <c r="C2" t="str">
-        <v>internal-support</v>
+        <v>A community of Python users across EMBL sharing knowledge and meetups.</v>
       </c>
       <c r="D2" t="str">
-        <v>Data Science Internal Support</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Book a one-to-one session with a data-science expert.</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
+        <v>https://bio-it.embl.de/embl-python-user-group/</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>bioimage-service</v>
+        <v>emblr</v>
       </c>
       <c r="B3" t="str">
-        <v>Bioimage analysis service</v>
+        <v>emblR</v>
       </c>
       <c r="C3" t="str">
-        <v>bioimage-analysis</v>
+        <v>The EMBL R user community, talks, help and code sharing for R users.</v>
       </c>
       <c r="D3" t="str">
-        <v>Bioimage Analysis Service</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Get help extracting quantitative data from your microscopy images.</v>
-      </c>
-      <c r="F3" t="str">
-        <v/>
+        <v>https://bio-it.embl.de/emblr/</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>data-management-support</v>
+        <v>workflows-club</v>
       </c>
       <c r="B4" t="str">
-        <v>Data management support</v>
+        <v>Scientific Workflows Club</v>
       </c>
       <c r="C4" t="str">
-        <v>data-management</v>
+        <v>Sharing experience building and running scientific workflows.</v>
       </c>
       <c r="D4" t="str">
-        <v>Data Management</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Plan, organise, document and share your research data (FAIR / RDM).</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
+        <v>https://docs.google.com/spreadsheets/d/1hI-NAJhP4OCQSAxM-oo-bwcM_6AuPlkzpCrkg4pND1I/edit?gid=0#gid=0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>training-courses</v>
+        <v>ai-reading-club</v>
       </c>
       <c r="B5" t="str">
-        <v>Training courses &amp; workshops</v>
+        <v>AI Reading Club</v>
       </c>
       <c r="C5" t="str">
-        <v>internal-support</v>
+        <v>Reading and discussing papers in AI and machine learning.</v>
       </c>
       <c r="D5" t="str">
-        <v>Data Science Internal Support</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Browse and sign up for data and software skills courses.</v>
-      </c>
-      <c r="F5" t="str">
-        <v/>
+        <v>https://chat.embl.org/embl/channels/ai-reading-club</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>infrastructure-access</v>
+        <v>bioinforome</v>
       </c>
       <c r="B6" t="str">
-        <v>Access to compute platforms</v>
+        <v>BioinfoRome</v>
       </c>
       <c r="C6" t="str">
-        <v>modis</v>
+        <v>The bioinformatics community at EMBL Rome.</v>
       </c>
       <c r="D6" t="str">
-        <v>Multimodal Open Data Integration Support</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Get access to JupyterHub, BAND, Galaxy and other shared platforms.</v>
-      </c>
-      <c r="F6" t="str">
-        <v/>
+        <v>https://chat.embl.org/embl/channels/bioinforome</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2150,16 +1935,16 @@
         <v>team_also_name</v>
       </c>
       <c r="I1" t="str">
+        <v>other_teams</v>
+      </c>
+      <c r="J1" t="str">
         <v>needs</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>people</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>why</v>
-      </c>
-      <c r="L1" t="str">
-        <v>difficulty</v>
       </c>
     </row>
     <row r="2">
@@ -2188,16 +1973,16 @@
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v>image-analysis</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
       </c>
-      <c r="K2" t="str">
-        <v>Counting cells across thousands of images is bread-and-butter bioimage analysis — and far kinder to your tendons.</v>
-      </c>
       <c r="L2" t="str">
-        <v>easy</v>
+        <v>Counting cells across thousands of images is bread-and-butter bioimage analysis, and far kinder to your tendons.</v>
       </c>
     </row>
     <row r="3">
@@ -2226,16 +2011,16 @@
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v>statistics</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Yuhong Liu</v>
       </c>
-      <c r="K3" t="str">
-        <v>Picking and interpreting the right statistical test is exactly what the internal support statisticians are for — before you commit to vibes.</v>
-      </c>
       <c r="L3" t="str">
-        <v>easy</v>
+        <v>Picking and interpreting the right statistical test is what the data science internal support statisticians are for, before you commit to vibes.</v>
       </c>
     </row>
     <row r="4">
@@ -2246,7 +2031,7 @@
         <v>staff</v>
       </c>
       <c r="C4" t="str">
-        <v>My analysis takes three days on my laptop, which is now also my space heater. Can we make it a real pipeline on the cluster?</v>
+        <v>My analysis takes three days on my laptop, which doubles as a space heater, not what I need during a heatwave! Can we make it a real pipeline on the cluster?</v>
       </c>
       <c r="D4" t="str">
         <v>yes</v>
@@ -2264,16 +2049,16 @@
         <v/>
       </c>
       <c r="I4" t="str">
+        <v>Data Management, Data Science Internal Support, Bioimage Analysis Service</v>
+      </c>
+      <c r="J4" t="str">
         <v>workflows</v>
       </c>
-      <c r="J4" t="str">
-        <v>Charles Girardot, Matthias Monfort, Laurent Thomas</v>
-      </c>
       <c r="K4" t="str">
-        <v>Turning a slow laptop script into a scalable, reproducible cluster workflow is MODIS / workflow-management territory.</v>
+        <v>Felix Schneider, Christian Tischer, Arif Ul Maula Khan, Yi Sun, Francesco Tabaro, Thomas Weber, Charles Girardot, Matthias Monfort, Laurent Thomas</v>
       </c>
       <c r="L4" t="str">
-        <v>easy</v>
+        <v>Turning a slow laptop script into a scalable, reproducible cluster workflow is data-science territory, which DSC team helps depends on your data and use case.</v>
       </c>
     </row>
     <row r="5">
@@ -2302,16 +2087,16 @@
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v>data-management</v>
       </c>
-      <c r="J5" t="str">
+      <c r="K5" t="str">
         <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
       </c>
-      <c r="K5" t="str">
-        <v>Structuring, documenting and sharing a lab's data is data-management work — frequently mistaken for an IT problem.</v>
-      </c>
       <c r="L5" t="str">
-        <v>boundary</v>
+        <v>Structuring, documenting and sharing a lab's data is data-management work, frequently mistaken for an IT problem.</v>
       </c>
     </row>
     <row r="6">
@@ -2340,16 +2125,16 @@
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
         <v>machine-learning, image-analysis</v>
       </c>
-      <c r="J6" t="str">
+      <c r="K6" t="str">
         <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
       </c>
-      <c r="K6" t="str">
-        <v>Training a model to classify phenotypes from images combines machine learning with bioimage analysis — both squarely DSC.</v>
-      </c>
       <c r="L6" t="str">
-        <v>easy</v>
+        <v>Training a model to classify phenotypes from images combines machine learning with bioimage analysis, two things the DSC handles every day.</v>
       </c>
     </row>
     <row r="7">
@@ -2360,7 +2145,7 @@
         <v>PI</v>
       </c>
       <c r="C7" t="str">
-        <v>How many biological replicates do I actually need — asking for the reviewer who will definitely complain about n=3?</v>
+        <v>How many biological replicates do I actually need, asking for the reviewer who will definitely complain about n=3?</v>
       </c>
       <c r="D7" t="str">
         <v>yes</v>
@@ -2378,16 +2163,16 @@
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v>statistics</v>
       </c>
-      <c r="J7" t="str">
+      <c r="K7" t="str">
         <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Yuhong Liu</v>
       </c>
-      <c r="K7" t="str">
-        <v>Replicate numbers are a power-analysis question for the statisticians — best asked before you run the experiment, not after the reviewer does.</v>
-      </c>
       <c r="L7" t="str">
-        <v>boundary</v>
+        <v>Replicate numbers are a power-analysis question for the statisticians, best asked before you run the experiment, not after the reviewer does.</v>
       </c>
     </row>
     <row r="8">
@@ -2416,16 +2201,16 @@
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
         <v>image-analysis</v>
       </c>
-      <c r="J8" t="str">
+      <c r="K8" t="str">
         <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
       </c>
-      <c r="K8" t="str">
+      <c r="L8" t="str">
         <v>Segmenting and measuring structures in 3D microscopy volumes is advanced image analysis.</v>
-      </c>
-      <c r="L8" t="str">
-        <v>easy</v>
       </c>
     </row>
     <row r="9">
@@ -2436,7 +2221,7 @@
         <v>fellow</v>
       </c>
       <c r="C9" t="str">
-        <v>My Python script works, technically — I just have time to make coffee, drink it, and regret things while it runs. Can someone speed it up?</v>
+        <v>My Python script works, technically, I just have time to make coffee, drink it, and regret things while it runs. Can someone speed it up?</v>
       </c>
       <c r="D9" t="str">
         <v>yes</v>
@@ -2454,16 +2239,16 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>workflows</v>
+        <v/>
       </c>
       <c r="J9" t="str">
-        <v>Felix Schneider</v>
+        <v>software</v>
       </c>
       <c r="K9" t="str">
-        <v>Profiling and optimising research code is research-software-engineering help from the internal support team.</v>
+        <v>Arif Ul Maula Khan, Leila Abbaspour, Tanuja Selvaraj, Thomas Weber, Matthias Monfort, Nayeem Reza, Laurent Thomas, Marco Wetter</v>
       </c>
       <c r="L9" t="str">
-        <v>boundary</v>
+        <v>Profiling and optimising research code is research-software-engineering help, and people across the DSC can dig into it depending on your stack.</v>
       </c>
     </row>
     <row r="10">
@@ -2492,16 +2277,16 @@
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>data-management</v>
+        <v/>
       </c>
       <c r="J10" t="str">
-        <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
+        <v>data-management, data-integration</v>
       </c>
       <c r="K10" t="str">
-        <v>Translating "community metadata standards" into actual ontologies and fields is exactly what the Data Management team does — so your data plays nicely with everyone else's.</v>
+        <v>Jean-Karim Hériché, Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez, Charles Girardot, Laurent Thomas</v>
       </c>
       <c r="L10" t="str">
-        <v>boundary</v>
+        <v>Translating "community metadata standards" into actual ontologies and fields is data-management and integration work, so your data plays nicely with everyone else's. Which DSC people help depends on your data.</v>
       </c>
     </row>
     <row r="11">
@@ -2530,16 +2315,16 @@
         <v/>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
         <v>data-management</v>
       </c>
-      <c r="J11" t="str">
-        <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
-      </c>
       <c r="K11" t="str">
-        <v>Writing the data management plan for a grant is a core data-management service — ideally before Friday.</v>
+        <v>Jean-Karim Hériché, Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez, Charles Girardot, Laurent Thomas</v>
       </c>
       <c r="L11" t="str">
-        <v>easy</v>
+        <v>Writing a data management plan for a grant is core data-management work, and people across the DSC (including bioimage analysis) can help, ideally before Friday.</v>
       </c>
     </row>
     <row r="12">
@@ -2568,16 +2353,16 @@
         <v/>
       </c>
       <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
         <v>training</v>
       </c>
-      <c r="J12" t="str">
+      <c r="K12" t="str">
         <v>Lisanna Paladin, Sarah Kaspar, Deborah Udoh, Eva-Maria Geissen, Felix Schneider, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves, Yuhong Liu</v>
       </c>
-      <c r="K12" t="str">
-        <v>Learning to code for data analysis is covered by the Data Science Centre's training offer — cake optional.</v>
-      </c>
       <c r="L12" t="str">
-        <v>easy</v>
+        <v>Learning to code for data analysis is covered by the Data Science Centre's training offer, cake optional.</v>
       </c>
     </row>
     <row r="13">
@@ -2606,16 +2391,16 @@
         <v/>
       </c>
       <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
         <v>software, training</v>
       </c>
-      <c r="J13" t="str">
+      <c r="K13" t="str">
         <v>Lisanna Paladin, Sarah Kaspar, Deborah Udoh, Eva-Maria Geissen, Felix Schneider, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves, Yuhong Liu</v>
       </c>
-      <c r="K13" t="str">
+      <c r="L13" t="str">
         <v>Setting up version control and sane software practice is research-software-engineering help from the internal support team.</v>
-      </c>
-      <c r="L13" t="str">
-        <v>boundary</v>
       </c>
     </row>
     <row r="14">
@@ -2626,7 +2411,7 @@
         <v>core-facility</v>
       </c>
       <c r="C14" t="str">
-        <v>I have a beautiful confocal stack and just need someone to count the fluorescent puncta per nucleus — automatically, for 500 images.</v>
+        <v>I have a beautiful confocal stack and just need someone to count the fluorescent puncta per nucleus, automatically, for 500 images.</v>
       </c>
       <c r="D14" t="str">
         <v>yes</v>
@@ -2644,16 +2429,16 @@
         <v/>
       </c>
       <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
         <v>image-analysis</v>
       </c>
-      <c r="J14" t="str">
+      <c r="K14" t="str">
         <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
       </c>
-      <c r="K14" t="str">
+      <c r="L14" t="str">
         <v>Automated puncta detection and per-nucleus quantification across hundreds of images is exactly what the Bioimage Analysis Service does.</v>
-      </c>
-      <c r="L14" t="str">
-        <v>easy</v>
       </c>
     </row>
     <row r="15">
@@ -2664,7 +2449,7 @@
         <v>fellow</v>
       </c>
       <c r="C15" t="str">
-        <v>I built an R Shiny app to explore our results and my collaborators keep asking me to "just send the link" — can someone host it properly instead of me leaving my laptop on overnight?</v>
+        <v>I built an R Shiny app to explore our results and my collaborators keep asking me to "just send the link", can someone host it properly instead of me leaving my laptop on overnight?</v>
       </c>
       <c r="D15" t="str">
         <v>yes</v>
@@ -2682,16 +2467,16 @@
         <v/>
       </c>
       <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
         <v>web, software</v>
       </c>
-      <c r="J15" t="str">
-        <v>Matthias Monfort, Nayeem Reza, Laurent Thomas, Marco Wetter</v>
-      </c>
       <c r="K15" t="str">
-        <v>Deploying and hosting containerised interactive apps (Shiny, dashboards) on EMBL infrastructure is MODIS's ShinyProxy territory — so your laptop can finally sleep.</v>
+        <v>Jean-Karim Hériché, Thomas Weber, Jacobo Miranda</v>
       </c>
       <c r="L15" t="str">
-        <v>boundary</v>
+        <v>Deploying and hosting containerised interactive apps (Shiny, dashboards) on EMBL infrastructure is a DSC job, so your laptop can finally sleep. It is not always the obvious team, the people who run this hosting span several teams.</v>
       </c>
     </row>
     <row r="16">
@@ -2720,16 +2505,16 @@
         <v/>
       </c>
       <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
         <v>data-management, data-integration</v>
       </c>
-      <c r="J16" t="str">
-        <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
-      </c>
       <c r="K16" t="str">
-        <v>Harmonising inconsistent metadata into one coherent, integrable schema is exactly what the Data Management team does — so "t0", "0h" and "baseline" finally mean the same thing.</v>
+        <v>Jean-Karim Hériché, Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez, Charles Girardot, Laurent Thomas</v>
       </c>
       <c r="L16" t="str">
-        <v>boundary</v>
+        <v>Harmonising inconsistent metadata into one coherent, integrable schema is data-management and integration work, so "t0", "0h" and "baseline" finally mean the same thing. Data Management leads, but they are not the only ones who can help.</v>
       </c>
     </row>
     <row r="17">
@@ -2740,7 +2525,7 @@
         <v>staff</v>
       </c>
       <c r="C17" t="str">
-        <v>My analysis pipeline runs perfectly on my machine and absolutely nowhere else — I'd like to containerise it so reviewers (and future me) can actually reproduce it.</v>
+        <v>My analysis pipeline runs perfectly on my machine and absolutely nowhere else, I'd like to containerise it so reviewers (and future me) can actually reproduce it.</v>
       </c>
       <c r="D17" t="str">
         <v>yes</v>
@@ -2758,16 +2543,16 @@
         <v/>
       </c>
       <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
         <v>workflows, software</v>
       </c>
-      <c r="J17" t="str">
-        <v>Charles Girardot, Matthias Monfort, Nayeem Reza, Laurent Thomas, Marco Wetter</v>
-      </c>
       <c r="K17" t="str">
-        <v>Containerising a pipeline for portability and reproducibility is core MODIS / workflow work — defeating the eternal "works on my machine" curse.</v>
+        <v>Renato Alves, Jean-Karim Hériché, Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez, Thomas Weber</v>
       </c>
       <c r="L17" t="str">
-        <v>boundary</v>
+        <v>Containerising a pipeline for portability and reproducibility is data-science workflow and software work, and several people across the DSC (MODIS, Data Management and beyond) can help, defeating the eternal "works on my machine" curse.</v>
       </c>
     </row>
     <row r="18">
@@ -2802,10 +2587,10 @@
         <v/>
       </c>
       <c r="K18" t="str">
-        <v>Buying and racking GPU hardware is IT. We (the DSC) design and train the model once the metal is humming — bring it to us then.</v>
+        <v/>
       </c>
       <c r="L18" t="str">
-        <v>boundary</v>
+        <v>Buying and racking GPU hardware is IT. We (the DSC) help you design and train the model once the metal is humming, bring it to us then.</v>
       </c>
     </row>
     <row r="19">
@@ -2840,10 +2625,10 @@
         <v/>
       </c>
       <c r="K19" t="str">
-        <v>Software licences and installation are IT's department — even when the software is pure data crunching. We can't conjure you a licence, sorry.</v>
+        <v/>
       </c>
       <c r="L19" t="str">
-        <v>boundary</v>
+        <v>Software licences and installation are IT's department, even when the software is pure data crunching. We can't conjure you a licence, sorry.</v>
       </c>
     </row>
     <row r="20">
@@ -2878,10 +2663,10 @@
         <v/>
       </c>
       <c r="K20" t="str">
-        <v>Storage capacity and network drives are IT's to grow. The DSC can later help you tidy and archive the mess — but the extra terabytes come from IT.</v>
+        <v/>
       </c>
       <c r="L20" t="str">
-        <v>boundary</v>
+        <v>Storage capacity and network drives are IT's to grow. The DSC can later help you tidy and archive the mess, but the extra terabytes come from IT.</v>
       </c>
     </row>
     <row r="21">
@@ -2892,7 +2677,7 @@
         <v>fellow</v>
       </c>
       <c r="C21" t="str">
-        <v>Working from home and I can't reach my data on the institute server — the VPN and I are not on speaking terms.</v>
+        <v>Working from home and I can't reach my data on the institute server, the VPN and I are not on speaking terms.</v>
       </c>
       <c r="D21" t="str">
         <v>no</v>
@@ -2916,10 +2701,10 @@
         <v/>
       </c>
       <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
         <v>Remote access and VPN wrangling are IT, not the Data Science Centre. Once you're connected, we're happy to talk data.</v>
-      </c>
-      <c r="L21" t="str">
-        <v>boundary</v>
       </c>
     </row>
     <row r="22">
@@ -2930,7 +2715,7 @@
         <v>fellow</v>
       </c>
       <c r="C22" t="str">
-        <v>GeneCore sequenced my 96 RNA libraries — now can the DSC demultiplex them, run FastQC, and hand me a tidy gene-count matrix?</v>
+        <v>GeneCore sequenced my 96 RNA libraries, now can the DSC demultiplex them, run FastQC, and hand me a tidy gene-count matrix?</v>
       </c>
       <c r="D22" t="str">
         <v>no</v>
@@ -2954,10 +2739,10 @@
         <v/>
       </c>
       <c r="K22" t="str">
-        <v>Demultiplexing, standard QC reports and a reference-aligned count matrix are GeneCore's standard primary processing, delivered bundled with the run. The DSC only takes over for the custom downstream — differential expression, odd designs, integration.</v>
+        <v/>
       </c>
       <c r="L22" t="str">
-        <v>boundary</v>
+        <v>Demultiplexing, standard QC reports and a reference-aligned count matrix are GeneCore's standard primary processing, delivered bundled with the run. The DSC only takes over for the custom downstream, differential expression, odd designs, integration.</v>
       </c>
     </row>
     <row r="23">
@@ -2992,10 +2777,10 @@
         <v/>
       </c>
       <c r="K23" t="str">
-        <v>UniProt is an EMBL-EBI public resource — that's where annotations live. The DSC isn't a lookup desk for public databases.</v>
+        <v/>
       </c>
       <c r="L23" t="str">
-        <v>easy</v>
+        <v>UniProt is an EMBL-EBI public resource, that's where annotations live. The DSC isn't a lookup desk for public databases.</v>
       </c>
     </row>
     <row r="24">
@@ -3027,13 +2812,13 @@
         <v/>
       </c>
       <c r="J24" t="str">
-        <v>Lisanna Paladin, Sarah Kaspar, Deborah Udoh, Eva-Maria Geissen, Felix Schneider, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves, Yuhong Liu</v>
+        <v>infrastructure</v>
       </c>
       <c r="K24" t="str">
-        <v>Come to the DSC first — we'll get you oriented and show you how to actually make the cluster do real analysis, then point you to IT, who own the accounts and SSH keys that unlock access.</v>
+        <v>Renato Alves, Yi Sun, Jean-Karim Hériché, Thomas Weber, Nayeem Reza, Marco Wetter</v>
       </c>
       <c r="L24" t="str">
-        <v>boundary</v>
+        <v>Come to the DSC first, we'll get you oriented and show you how to actually make the cluster do real analysis, then point you to IT, who own the accounts and SSH keys that unlock access.</v>
       </c>
     </row>
     <row r="25">
@@ -3062,16 +2847,16 @@
         <v>IT Services</v>
       </c>
       <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
         <v>data-management</v>
       </c>
-      <c r="J25" t="str">
+      <c r="K25" t="str">
         <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
       </c>
-      <c r="K25" t="str">
-        <v>Start with the DSC's Data Management team — they advise which database to pick and design a FAIR schema so it isn't chaos. IT then hosts and maintains the actual server (a VM or Kubernetes DB operator).</v>
-      </c>
       <c r="L25" t="str">
-        <v>boundary</v>
+        <v>Start with the DSC's Data Management team, they advise which database to pick and design a FAIR schema so it isn't chaos. IT then hosts and maintains the actual server (a VM or Kubernetes DB operator).</v>
       </c>
     </row>
     <row r="26">
@@ -3103,13 +2888,13 @@
         <v/>
       </c>
       <c r="J26" t="str">
-        <v>Lisanna Paladin, Sarah Kaspar, Deborah Udoh, Eva-Maria Geissen, Felix Schneider, Isabela Paredes-Cisneros, Jacobo Miranda, Renato Alves, Yuhong Liu</v>
+        <v/>
       </c>
       <c r="K26" t="str">
+        <v>Renato Alves</v>
+      </c>
+      <c r="L26" t="str">
         <v>The DSC runs and governs the JupyterHub service, so come to us first when it falls over. IT provides the underlying infrastructure it sits on.</v>
-      </c>
-      <c r="L26" t="str">
-        <v>boundary</v>
       </c>
     </row>
     <row r="27">
@@ -3138,16 +2923,16 @@
         <v>IT Services</v>
       </c>
       <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
         <v>data-management</v>
       </c>
-      <c r="J27" t="str">
+      <c r="K27" t="str">
         <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
       </c>
-      <c r="K27" t="str">
+      <c r="L27" t="str">
         <v>Start with the DSC's Data Management team to plan what's worth keeping and how to preserve and share it long-term. IT then runs the backup infrastructure that copies your bytes.</v>
-      </c>
-      <c r="L27" t="str">
-        <v>boundary</v>
       </c>
     </row>
     <row r="28">
@@ -3176,16 +2961,16 @@
         <v>Core Facilities</v>
       </c>
       <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
         <v>workflows, data-management</v>
       </c>
-      <c r="J28" t="str">
+      <c r="K28" t="str">
         <v>Charles Girardot, Matthias Monfort, Laurent Thomas</v>
       </c>
-      <c r="K28" t="str">
+      <c r="L28" t="str">
         <v>Core Facilities deliver the raw reads; MODIS builds the scalable, reproducible pipeline to turn them into results. Two stops, one happy genomicist.</v>
-      </c>
-      <c r="L28" t="str">
-        <v>boundary</v>
       </c>
     </row>
     <row r="29">
@@ -3196,7 +2981,7 @@
         <v>staff</v>
       </c>
       <c r="C29" t="str">
-        <v>My 40 protein samples are off the mass spec — can you run a MaxQuant search and give me identified, quantified proteins? Sounds like a proteomics-bioinformatics job, right?</v>
+        <v>My 40 protein samples are off the mass spec, can you run a MaxQuant search and give me identified, quantified proteins? Sounds like a proteomics-bioinformatics job, right?</v>
       </c>
       <c r="D29" t="str">
         <v>shared</v>
@@ -3214,16 +2999,16 @@
         <v>Core Facilities</v>
       </c>
       <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
         <v>statistics, workflows</v>
       </c>
-      <c r="J29" t="str">
+      <c r="K29" t="str">
         <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Yuhong Liu</v>
       </c>
-      <c r="K29" t="str">
-        <v>A standard MaxQuant identification-and-quantification search is actually the Proteomics Core Facility's bundled service. Start with the DSC and we'll point you there for the standard search, then pick up the custom bit — bespoke statistics and a reproducible downstream workflow.</v>
-      </c>
       <c r="L29" t="str">
-        <v>boundary</v>
+        <v>A standard MaxQuant identification-and-quantification search is actually the Proteomics Core Facility's bundled service. Start with the DSC and we'll point you there for the standard search, then pick up the custom bit, bespoke statistics and a reproducible downstream workflow.</v>
       </c>
     </row>
     <row r="30">
@@ -3234,7 +3019,7 @@
         <v>staff</v>
       </c>
       <c r="C30" t="str">
-        <v>My paper's in review and I need to deposit my transcriptomics data in a public archive — which one, and how do I make it FAIR?</v>
+        <v>My paper's in review and I need to deposit my transcriptomics data in a public archive, which one, and how do I make it FAIR?</v>
       </c>
       <c r="D30" t="str">
         <v>shared</v>
@@ -3252,16 +3037,16 @@
         <v>EMBL-EBI</v>
       </c>
       <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
         <v>data-management</v>
       </c>
-      <c r="J30" t="str">
+      <c r="K30" t="str">
         <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
       </c>
-      <c r="K30" t="str">
+      <c r="L30" t="str">
         <v>Data Management helps you pick the right repository and make the data FAIR; EMBL-EBI hosts the archive (e.g. ArrayExpress) that actually stores it. Talk to us first.</v>
-      </c>
-      <c r="L30" t="str">
-        <v>boundary</v>
       </c>
     </row>
     <row r="31">
@@ -3272,10 +3057,10 @@
         <v>PI</v>
       </c>
       <c r="C31" t="str">
-        <v>My core-facility output is great but my lab can't explore it — I want a pipeline that feeds an interactive dashboard everyone can click through.</v>
+        <v>My core-facility output is great but my lab can't explore it, I want a pipeline that feeds an interactive dashboard everyone can click through.</v>
       </c>
       <c r="D31" t="str">
-        <v>shared</v>
+        <v>yes</v>
       </c>
       <c r="E31" t="str">
         <v>modis</v>
@@ -3284,22 +3069,22 @@
         <v>Multimodal Open Data Integration Support</v>
       </c>
       <c r="G31" t="str">
-        <v>internal-support</v>
+        <v/>
       </c>
       <c r="H31" t="str">
-        <v>Data Science Internal Support</v>
+        <v/>
       </c>
       <c r="I31" t="str">
-        <v>workflows, software</v>
+        <v/>
       </c>
       <c r="J31" t="str">
-        <v>Charles Girardot, Matthias Monfort, Nayeem Reza, Laurent Thomas, Marco Wetter</v>
+        <v>workflows, software, web</v>
       </c>
       <c r="K31" t="str">
-        <v>MODIS wires the workflow into a deployable dashboard; Internal Support's RSEs help polish and maintain the app. Goodbye, screenshots pasted into Mattermost.</v>
+        <v>Thomas Weber, Jean-Karim Hériché, Jacobo Miranda</v>
       </c>
       <c r="L31" t="str">
-        <v>hard</v>
+        <v>The DSC wires your workflow into a deployable dashboard and helps polish and maintain the app, and which people help depends on your stack. Goodbye, screenshots pasted into Mattermost.</v>
       </c>
     </row>
     <row r="32">
@@ -3310,7 +3095,7 @@
         <v>fellow</v>
       </c>
       <c r="C32" t="str">
-        <v>Metabolomics ran my samples and gave me annotated compounds, but now I want to correlate those metabolite levels against my custom drug-dose design — can the DSC crunch that?</v>
+        <v>Metabolomics CF ran my samples and gave me annotated compounds, but now I want to correlate those metabolite levels against my custom drug-dose design, can the DSC crunch that?</v>
       </c>
       <c r="D32" t="str">
         <v>shared</v>
@@ -3328,16 +3113,16 @@
         <v>Core Facilities</v>
       </c>
       <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
         <v>statistics</v>
       </c>
-      <c r="J32" t="str">
+      <c r="K32" t="str">
         <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Yuhong Liu</v>
       </c>
-      <c r="K32" t="str">
-        <v>Standard compound annotation is the Metabolomics Core Facility's bundled deliverable, so start with the DSC and we'll confirm that part lives there — then we pick up the custom downstream, the dose-response statistics and correlation analysis.</v>
-      </c>
       <c r="L32" t="str">
-        <v>boundary</v>
+        <v>Standard compound annotation is the Metabolomics Core Facility's bundled deliverable, so start with the DSC and we'll confirm that part lives there, then we pick up the custom downstream, the dose-response statistics and correlation analysis.</v>
       </c>
     </row>
     <row r="33">
@@ -3348,7 +3133,7 @@
         <v>core-facility</v>
       </c>
       <c r="C33" t="str">
-        <v>Flow Cytometry already gated my populations the standard way — now I want an unsupervised clustering and trajectory analysis across 80 samples to find a subset nobody's drawn a gate around yet.</v>
+        <v>Flow Cytometry already gated my populations the standard way, now I want an unsupervised clustering and trajectory analysis across 80 samples to find a subset nobody's drawn a gate around yet.</v>
       </c>
       <c r="D33" t="str">
         <v>shared</v>
@@ -3366,16 +3151,16 @@
         <v>Core Facilities</v>
       </c>
       <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
         <v>statistics, machine-learning</v>
       </c>
-      <c r="J33" t="str">
+      <c r="K33" t="str">
         <v>Sarah Kaspar, Eva-Maria Geissen, Felix Schneider, Jacobo Miranda, Yuhong Liu</v>
       </c>
-      <c r="K33" t="str">
-        <v>Standard gating is the Flow Cytometry Core Facility's job; the DSC takes over for the custom bit — unsupervised clustering and high-dimensional analysis that no manual gate can capture. Talk to us first for the downstream.</v>
-      </c>
       <c r="L33" t="str">
-        <v>boundary</v>
+        <v>Standard gating is the Flow Cytometry Core Facility's job; the DSC takes over for the custom bit, unsupervised clustering and high-dimensional analysis that no manual gate can capture. Talk to us first for the downstream.</v>
       </c>
     </row>
     <row r="34">
@@ -3386,10 +3171,10 @@
         <v>staff</v>
       </c>
       <c r="C34" t="str">
-        <v>The Light Microscopy facility deconvolved and stitched my big tiled acquisition beautifully — now I need a custom pipeline to quantify membrane-to-cytoplasm ratios per cell across the whole mosaic.</v>
+        <v>The Light Microscopy facility deconvolved and stitched my big tiled acquisition beautifully, now I need a custom pipeline to quantify membrane-to-cytoplasm ratios per cell across the whole mosaic.</v>
       </c>
       <c r="D34" t="str">
-        <v>shared</v>
+        <v>yes</v>
       </c>
       <c r="E34" t="str">
         <v>bioimage-analysis</v>
@@ -3398,22 +3183,22 @@
         <v>Bioimage Analysis Service</v>
       </c>
       <c r="G34" t="str">
-        <v>core-facilities</v>
+        <v/>
       </c>
       <c r="H34" t="str">
-        <v>Core Facilities</v>
+        <v/>
       </c>
       <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
         <v>image-analysis</v>
       </c>
-      <c r="J34" t="str">
+      <c r="K34" t="str">
         <v>Christian Tischer, Arif Ul Maula Khan, Yi Sun, Jean-Karim Hériché, Leila Abbaspour</v>
       </c>
-      <c r="K34" t="str">
-        <v>Acquisition, deconvolution and stitching are the facility's standard processing; bespoke per-cell quantification is DSC bioimage analysis. Come to us first for the custom measurement, then the facility for any reacquisition.</v>
-      </c>
       <c r="L34" t="str">
-        <v>boundary</v>
+        <v>The facility already did the acquisition, deconvolution and stitching. Building a custom pipeline to quantify membrane-to-cytoplasm ratios per cell across the mosaic is DSC bioimage analysis.</v>
       </c>
     </row>
     <row r="35">
@@ -3442,16 +3227,16 @@
         <v>Data Management</v>
       </c>
       <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
         <v>data-management</v>
       </c>
-      <c r="J35" t="str">
+      <c r="K35" t="str">
         <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
       </c>
-      <c r="K35" t="str">
-        <v>IT first — they own the secure large-file transfer (Aspera/Globus) that actually moves 8 TB across the planet. The DSC's Data Management team then helps structure and document what arrives so it isn't 8 TB of mystery.</v>
-      </c>
       <c r="L35" t="str">
-        <v>boundary</v>
+        <v>IT first, they own the secure large-file transfer (Aspera/Globus) that actually moves 8 TB across the planet. The DSC's Data Management team then helps structure and document what arrives so it isn't 8 TB of mystery.</v>
       </c>
     </row>
     <row r="36">
@@ -3480,16 +3265,16 @@
         <v>Data Management</v>
       </c>
       <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
         <v>data-management</v>
       </c>
-      <c r="J36" t="str">
+      <c r="K36" t="str">
         <v>Erick Martins Ratamero, Tanuja Selvaraj, Francesco Tabaro, Nora Vivanco Gonzalez</v>
       </c>
-      <c r="K36" t="str">
+      <c r="L36" t="str">
         <v>Moving data between EMBL sites runs on IT's inter-site transfer infrastructure, so go to IT first. The DSC's Data Management team helps organise and document the dataset so the copy at the other end makes sense.</v>
-      </c>
-      <c r="L36" t="str">
-        <v>boundary</v>
       </c>
     </row>
   </sheetData>

</xml_diff>